<commit_message>
FEAT: sync all track-history to NAS deep store (NAS-HISTORY-SYNC)
Only ticker_snapshots lived on the NAS; the precious histories (signal_log,
audit_ledger, picks_history, ml_edge) existed ONLY on the local Mac — so the NAS
wasn't yet a true backup. Now mirrored as schema-flexible JSONB archive tables:

- nas_pg.archive_json(): JSONB archive with NaN/Inf->null sanitize + in-batch
  key dedup (execute_values + ON CONFLICT can't touch a key twice).
- scripts/sync_history_to_nas.py: signal_log_archive 4713, audit_ledger_archive
  4915, picks_trades_archive 1766, picks_runs_archive 57, ml_edge_archive 1905.
- scripts/nas_sync_all.sh runs snapshots + history nightly via com.swingtrade.nas-sync.

NAS deep store now holds 209,630 rows across 6 tables — full track-history backup,
queryable from Postgres. Local files are no longer the only copy.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-06-18.xlsx
+++ b/cache/open_items_2026-06-18.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N312"/>
+  <dimension ref="A1:N313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -14848,13 +14848,13 @@
         </is>
       </c>
     </row>
-    <row r="259" ht="90" customHeight="1">
+    <row r="259" ht="75" customHeight="1">
       <c r="A259" s="2" t="n">
         <v>258</v>
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>NAS-PG-DEEP-STORE</t>
+          <t>NAS-HISTORY-SYNC</t>
         </is>
       </c>
       <c r="C259" s="10" t="inlineStr">
@@ -14869,17 +14869,17 @@
       </c>
       <c r="E259" s="6" t="inlineStr">
         <is>
-          <t>Self-hosted Postgres on Synology NAS as deep audit/snapshot store</t>
+          <t>Sync all track-history to NAS deep store</t>
         </is>
       </c>
       <c r="F259" s="5" t="inlineStr">
         <is>
-          <t>Local SQLite limited by 162GB-free disk (89% full); full snapshot retention untenable locally. Owner has DS1520+ NAS</t>
+          <t>Only ticker_snapshots was on NAS; signal_log/audit_ledger/picks_history/ml_edge existed only locally — not a true backup</t>
         </is>
       </c>
       <c r="G259" s="5" t="inlineStr">
         <is>
-          <t>Postgres 16 container on DS1520+ (192.168.1.25:5433); nas_pg.py (conn+schema+upsert), scripts/sync_snapshots_to_nas.py (idempotent push), ticker_snapshots.capture_scan best-effort real-time push, nightly catch-up launchd com.swingtrade.nas-sync. SQLite=hot 90d, NAS=full retention. 196K rows synced, raw_gz round-trips 292 fields. NAS_PG_URL in .env (gitignored)</t>
+          <t>nas_pg.archive_json (JSONB archive, NaN-sanitized, in-batch dedup); scripts/sync_history_to_nas.py mirrors signal_log(4713)/audit_ledger(4915)/picks_trades(1766)/picks_runs(57)/ml_edge(1905); nightly via scripts/nas_sync_all.sh in com.swingtrade.nas-sync; 209,630 total rows on NAS</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr"/>
@@ -14897,7 +14897,7 @@
       </c>
       <c r="M259" s="3" t="inlineStr">
         <is>
-          <t>76cca4dbd</t>
+          <t>cb4ef7114</t>
         </is>
       </c>
       <c r="N259" s="8" t="inlineStr"/>
@@ -14908,7 +14908,7 @@
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>UI-MLEDGE-1</t>
+          <t>NAS-PG-DEEP-STORE</t>
         </is>
       </c>
       <c r="C260" s="10" t="inlineStr">
@@ -14918,22 +14918,22 @@
       </c>
       <c r="D260" s="5" t="inlineStr">
         <is>
-          <t>ML Edge Tab</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E260" s="6" t="inlineStr">
         <is>
-          <t>Theme switching + tf-* visual port</t>
+          <t>Self-hosted Postgres on Synology NAS as deep audit/snapshot store</t>
         </is>
       </c>
       <c r="F260" s="5" t="inlineStr">
         <is>
-          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
+          <t>Local SQLite limited by 162GB-free disk (89% full); full snapshot retention untenable locally. Owner has DS1520+ NAS</t>
         </is>
       </c>
       <c r="G260" s="5" t="inlineStr">
         <is>
-          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
+          <t>Postgres 16 container on DS1520+ (192.168.1.25:5433); nas_pg.py (conn+schema+upsert), scripts/sync_snapshots_to_nas.py (idempotent push), ticker_snapshots.capture_scan best-effort real-time push, nightly catch-up launchd com.swingtrade.nas-sync. SQLite=hot 90d, NAS=full retention. 196K rows synced, raw_gz round-trips 292 fields. NAS_PG_URL in .env (gitignored)</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr"/>
@@ -14946,23 +14946,23 @@
       </c>
       <c r="L260" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="M260" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
+          <t>76cca4dbd</t>
         </is>
       </c>
       <c r="N260" s="8" t="inlineStr"/>
     </row>
-    <row r="261" ht="45" customHeight="1">
+    <row r="261" ht="90" customHeight="1">
       <c r="A261" s="2" t="n">
         <v>260</v>
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>IPAD-2</t>
+          <t>UI-MLEDGE-1</t>
         </is>
       </c>
       <c r="C261" s="10" t="inlineStr">
@@ -14972,39 +14972,27 @@
       </c>
       <c r="D261" s="5" t="inlineStr">
         <is>
-          <t>Mobile / iPad</t>
+          <t>ML Edge Tab</t>
         </is>
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
+          <t>Theme switching + tf-* visual port</t>
         </is>
       </c>
       <c r="F261" s="5" t="inlineStr">
         <is>
-          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
+          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
         </is>
       </c>
       <c r="G261" s="5" t="inlineStr">
         <is>
-          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
-        </is>
-      </c>
-      <c r="H261" s="2" t="inlineStr">
-        <is>
-          <t>15 min</t>
-        </is>
-      </c>
-      <c r="I261" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J261" s="5" t="inlineStr">
-        <is>
-          <t>Sub-task of IPAD-1.</t>
-        </is>
-      </c>
+          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
+        </is>
+      </c>
+      <c r="H261" s="2" t="inlineStr"/>
+      <c r="I261" s="5" t="inlineStr"/>
+      <c r="J261" s="5" t="inlineStr"/>
       <c r="K261" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15012,19 +15000,15 @@
       </c>
       <c r="L261" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M261" s="3" t="inlineStr">
         <is>
-          <t>79fa01a75</t>
-        </is>
-      </c>
-      <c r="N261" s="8" t="inlineStr">
-        <is>
-          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
-        </is>
-      </c>
+          <t>696731a4d</t>
+        </is>
+      </c>
+      <c r="N261" s="8" t="inlineStr"/>
     </row>
     <row r="262" ht="45" customHeight="1">
       <c r="A262" s="2" t="n">
@@ -15032,7 +15016,7 @@
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>SLACK-NEWSLETTER-MLALERT</t>
+          <t>IPAD-2</t>
         </is>
       </c>
       <c r="C262" s="10" t="inlineStr">
@@ -15042,27 +15026,39 @@
       </c>
       <c r="D262" s="5" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile / iPad</t>
         </is>
       </c>
       <c r="E262" s="6" t="inlineStr">
         <is>
-          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
+          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
         </is>
       </c>
       <c r="F262" s="5" t="inlineStr">
         <is>
-          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
+          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
         </is>
       </c>
       <c r="G262" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd + scripts/ml_alert_slack.py</t>
-        </is>
-      </c>
-      <c r="H262" s="2" t="inlineStr"/>
-      <c r="I262" s="5" t="inlineStr"/>
-      <c r="J262" s="5" t="inlineStr"/>
+          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="I262" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J262" s="5" t="inlineStr">
+        <is>
+          <t>Sub-task of IPAD-1.</t>
+        </is>
+      </c>
       <c r="K262" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15070,15 +15066,19 @@
       </c>
       <c r="L262" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M262" s="3" t="inlineStr">
         <is>
-          <t>d1ea97913</t>
-        </is>
-      </c>
-      <c r="N262" s="8" t="inlineStr"/>
+          <t>79fa01a75</t>
+        </is>
+      </c>
+      <c r="N262" s="8" t="inlineStr">
+        <is>
+          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
+        </is>
+      </c>
     </row>
     <row r="263" ht="45" customHeight="1">
       <c r="A263" s="2" t="n">
@@ -15086,7 +15086,7 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>FORENSICS-WEEKLY-SLACK</t>
+          <t>SLACK-NEWSLETTER-MLALERT</t>
         </is>
       </c>
       <c r="C263" s="10" t="inlineStr">
@@ -15096,22 +15096,22 @@
       </c>
       <c r="D263" s="5" t="inlineStr">
         <is>
-          <t>Notifications / Audit</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>Weekly pick-forensics Slack digest</t>
+          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
         </is>
       </c>
       <c r="F263" s="5" t="inlineStr">
         <is>
-          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
+          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
         </is>
       </c>
       <c r="G263" s="5" t="inlineStr">
         <is>
-          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+          <t>infra/launchd + scripts/ml_alert_slack.py</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr"/>
@@ -15129,18 +15129,18 @@
       </c>
       <c r="M263" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d1ea97913</t>
         </is>
       </c>
       <c r="N263" s="8" t="inlineStr"/>
     </row>
-    <row r="264" ht="75" customHeight="1">
+    <row r="264" ht="45" customHeight="1">
       <c r="A264" s="2" t="n">
         <v>263</v>
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
+          <t>FORENSICS-WEEKLY-SLACK</t>
         </is>
       </c>
       <c r="C264" s="10" t="inlineStr">
@@ -15150,39 +15150,27 @@
       </c>
       <c r="D264" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Notifications / Audit</t>
         </is>
       </c>
       <c r="E264" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Weekly pick-forensics Slack digest</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
         </is>
       </c>
       <c r="G264" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
-        </is>
-      </c>
-      <c r="H264" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I264" s="5" t="inlineStr">
-        <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
-        </is>
-      </c>
-      <c r="J264" s="5" t="inlineStr">
-        <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
-        </is>
-      </c>
+          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+        </is>
+      </c>
+      <c r="H264" s="2" t="inlineStr"/>
+      <c r="I264" s="5" t="inlineStr"/>
+      <c r="J264" s="5" t="inlineStr"/>
       <c r="K264" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15190,27 +15178,23 @@
       </c>
       <c r="L264" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M264" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N264" s="8" t="inlineStr">
-        <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="265" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N264" s="8" t="inlineStr"/>
+    </row>
+    <row r="265" ht="75" customHeight="1">
       <c r="A265" s="2" t="n">
         <v>264</v>
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C265" s="10" t="inlineStr">
@@ -15220,37 +15204,37 @@
       </c>
       <c r="D265" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E265" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F265" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G265" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I265" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J265" s="5" t="inlineStr">
         <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K265" s="12" t="inlineStr">
@@ -15260,17 +15244,17 @@
       </c>
       <c r="L265" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M265" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N265" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
         </is>
       </c>
     </row>
@@ -15280,7 +15264,7 @@
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C266" s="10" t="inlineStr">
@@ -15295,32 +15279,32 @@
       </c>
       <c r="E266" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F266" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G266" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I266" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J266" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K266" s="12" t="inlineStr">
@@ -15340,7 +15324,7 @@
       </c>
       <c r="N266" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -15350,7 +15334,7 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C267" s="10" t="inlineStr">
@@ -15365,32 +15349,32 @@
       </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F267" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G267" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I267" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J267" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K267" s="12" t="inlineStr">
@@ -15410,7 +15394,7 @@
       </c>
       <c r="N267" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
         </is>
       </c>
     </row>
@@ -15420,7 +15404,7 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>OPS-4</t>
         </is>
       </c>
       <c r="C268" s="10" t="inlineStr">
@@ -15435,32 +15419,32 @@
       </c>
       <c r="E268" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F268" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G268" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I268" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J268" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K268" s="12" t="inlineStr">
@@ -15470,27 +15454,27 @@
       </c>
       <c r="L268" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M268" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N268" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="269" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="269" ht="60" customHeight="1">
       <c r="A269" s="2" t="n">
         <v>268</v>
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>SCAN-FAILURE-ALERT</t>
+          <t>OPS-5</t>
         </is>
       </c>
       <c r="C269" s="10" t="inlineStr">
@@ -15500,27 +15484,39 @@
       </c>
       <c r="D269" s="5" t="inlineStr">
         <is>
-          <t>Ops / Alerts</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E269" s="6" t="inlineStr">
         <is>
-          <t>Scan-failure + EODHD-quota Slack alert</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F269" s="5" t="inlineStr">
         <is>
-          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G269" s="5" t="inlineStr">
         <is>
-          <t>swing_trade.py exit hook</t>
-        </is>
-      </c>
-      <c r="H269" s="2" t="inlineStr"/>
-      <c r="I269" s="5" t="inlineStr"/>
-      <c r="J269" s="5" t="inlineStr"/>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+        </is>
+      </c>
+      <c r="H269" s="2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I269" s="5" t="inlineStr">
+        <is>
+          <t>Win: fast iteration on report templates.</t>
+        </is>
+      </c>
+      <c r="J269" s="5" t="inlineStr">
+        <is>
+          <t>Trivial CLI wrapper.</t>
+        </is>
+      </c>
       <c r="K269" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15528,15 +15524,19 @@
       </c>
       <c r="L269" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr">
         <is>
-          <t>0dc7675ee</t>
-        </is>
-      </c>
-      <c r="N269" s="8" t="inlineStr"/>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N269" s="8" t="inlineStr">
+        <is>
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="270" ht="45" customHeight="1">
       <c r="A270" s="2" t="n">
@@ -15544,7 +15544,7 @@
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
+          <t>SCAN-FAILURE-ALERT</t>
         </is>
       </c>
       <c r="C270" s="10" t="inlineStr">
@@ -15554,22 +15554,22 @@
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Alerts</t>
         </is>
       </c>
       <c r="E270" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot: load or retire</t>
+          <t>Scan-failure + EODHD-quota Slack alert</t>
         </is>
       </c>
       <c r="F270" s="5" t="inlineStr">
         <is>
-          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
+          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
         </is>
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd</t>
+          <t>swing_trade.py exit hook</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr"/>
@@ -15592,13 +15592,13 @@
       </c>
       <c r="N270" s="8" t="inlineStr"/>
     </row>
-    <row r="271" ht="60" customHeight="1">
+    <row r="271" ht="45" customHeight="1">
       <c r="A271" s="2" t="n">
         <v>270</v>
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>OVERVIEW-TQ-LABEL</t>
+          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
         </is>
       </c>
       <c r="C271" s="10" t="inlineStr">
@@ -15608,22 +15608,22 @@
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
+          <t>Decide momentum-snapshot: load or retire</t>
         </is>
       </c>
       <c r="F271" s="5" t="inlineStr">
         <is>
-          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
+          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
         </is>
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
+          <t>infra/launchd</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr"/>
@@ -15636,23 +15636,23 @@
       </c>
       <c r="L271" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M271" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>0dc7675ee</t>
         </is>
       </c>
       <c r="N271" s="8" t="inlineStr"/>
     </row>
-    <row r="272" ht="150" customHeight="1">
+    <row r="272" ht="60" customHeight="1">
       <c r="A272" s="2" t="n">
         <v>271</v>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>OVERVIEW-TQ-LABEL</t>
         </is>
       </c>
       <c r="C272" s="10" t="inlineStr">
@@ -15662,31 +15662,27 @@
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="E272" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
         </is>
       </c>
       <c r="G272" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr"/>
       <c r="I272" s="5" t="inlineStr"/>
-      <c r="J272" s="5" t="inlineStr">
-        <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
-        </is>
-      </c>
+      <c r="J272" s="5" t="inlineStr"/>
       <c r="K272" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15694,27 +15690,23 @@
       </c>
       <c r="L272" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M272" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
-        </is>
-      </c>
-      <c r="N272" s="8" t="inlineStr">
-        <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="273" ht="105" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N272" s="8" t="inlineStr"/>
+    </row>
+    <row r="273" ht="150" customHeight="1">
       <c r="A273" s="2" t="n">
         <v>272</v>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>SMC-OB-DISPLAY-1</t>
+          <t>PERF-7b</t>
         </is>
       </c>
       <c r="C273" s="10" t="inlineStr">
@@ -15724,27 +15716,31 @@
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E273" s="6" t="inlineStr">
         <is>
-          <t>OB confluence badges in SMC tab</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F273" s="5" t="inlineStr">
         <is>
-          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G273" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr"/>
       <c r="I273" s="5" t="inlineStr"/>
-      <c r="J273" s="5" t="inlineStr"/>
+      <c r="J273" s="5" t="inlineStr">
+        <is>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+        </is>
+      </c>
       <c r="K273" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15752,23 +15748,27 @@
       </c>
       <c r="L273" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr">
         <is>
-          <t>8182c3977</t>
-        </is>
-      </c>
-      <c r="N273" s="8" t="inlineStr"/>
-    </row>
-    <row r="274" ht="75" customHeight="1">
+          <t>cf30df858</t>
+        </is>
+      </c>
+      <c r="N273" s="8" t="inlineStr">
+        <is>
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="274" ht="105" customHeight="1">
       <c r="A274" s="2" t="n">
         <v>273</v>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-COMPANY-NAMES</t>
+          <t>SMC-OB-DISPLAY-1</t>
         </is>
       </c>
       <c r="C274" s="10" t="inlineStr">
@@ -15778,22 +15778,22 @@
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Scanner UI</t>
+          <t>SMC</t>
         </is>
       </c>
       <c r="E274" s="6" t="inlineStr">
         <is>
-          <t>NAME column duplicated TICKER (no company names)</t>
+          <t>OB confluence badges in SMC tab</t>
         </is>
       </c>
       <c r="F274" s="5" t="inlineStr">
         <is>
-          <t>Scan feed set name=ticker; no cached name source (fundamentals.db raw_json has 0 names). NAME column was redundant.</t>
+          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
         </is>
       </c>
       <c r="G274" s="5" t="inlineStr">
         <is>
-          <t>Free Wikipedia S&amp;P1500+NDX+Dow name map (scripts/build_ticker_names.py -&gt; cache/ticker_names.json, 1508 names); joined in /api/universe _ticker_names(); weekly refresh in weekly_diagnostics.sh. 70% live coverage, honest ticker fallback for the tail. No paid data.</t>
+          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr"/>
@@ -15806,23 +15806,23 @@
       </c>
       <c r="L274" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr">
         <is>
-          <t>48f6a2fbf</t>
+          <t>8182c3977</t>
         </is>
       </c>
       <c r="N274" s="8" t="inlineStr"/>
     </row>
-    <row r="275" ht="45" customHeight="1">
+    <row r="275" ht="75" customHeight="1">
       <c r="A275" s="2" t="n">
         <v>274</v>
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-1</t>
+          <t>SCANNER-COMPANY-NAMES</t>
         </is>
       </c>
       <c r="C275" s="10" t="inlineStr">
@@ -15832,22 +15832,22 @@
       </c>
       <c r="D275" s="5" t="inlineStr">
         <is>
-          <t>Sharpe Roadmap</t>
+          <t>Scanner UI</t>
         </is>
       </c>
       <c r="E275" s="6" t="inlineStr">
         <is>
-          <t>Sharpe gate in momentum detector</t>
+          <t>NAME column duplicated TICKER (no company names)</t>
         </is>
       </c>
       <c r="F275" s="5" t="inlineStr">
         <is>
-          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
+          <t>Scan feed set name=ticker; no cached name source (fundamentals.db raw_json has 0 names). NAME column was redundant.</t>
         </is>
       </c>
       <c r="G275" s="5" t="inlineStr">
         <is>
-          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
+          <t>Free Wikipedia S&amp;P1500+NDX+Dow name map (scripts/build_ticker_names.py -&gt; cache/ticker_names.json, 1508 names); joined in /api/universe _ticker_names(); weekly refresh in weekly_diagnostics.sh. 70% live coverage, honest ticker fallback for the tail. No paid data.</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr"/>
@@ -15860,12 +15860,12 @@
       </c>
       <c r="L275" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr">
         <is>
-          <t>dbbd6b5f6</t>
+          <t>48f6a2fbf</t>
         </is>
       </c>
       <c r="N275" s="8" t="inlineStr"/>
@@ -15876,7 +15876,7 @@
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-10</t>
+          <t>SHARPE-1</t>
         </is>
       </c>
       <c r="C276" s="10" t="inlineStr">
@@ -15891,17 +15891,17 @@
       </c>
       <c r="E276" s="6" t="inlineStr">
         <is>
-          <t>Sharpe alerts for watchlist</t>
+          <t>Sharpe gate in momentum detector</t>
         </is>
       </c>
       <c r="F276" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
         </is>
       </c>
       <c r="G276" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
+          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr"/>
@@ -15930,7 +15930,7 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-11</t>
+          <t>SHARPE-10</t>
         </is>
       </c>
       <c r="C277" s="10" t="inlineStr">
@@ -15945,17 +15945,17 @@
       </c>
       <c r="E277" s="6" t="inlineStr">
         <is>
-          <t>Per-trade Sharpe attribution</t>
+          <t>Sharpe alerts for watchlist</t>
         </is>
       </c>
       <c r="F277" s="5" t="inlineStr">
         <is>
-          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G277" s="5" t="inlineStr">
         <is>
-          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
+          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr"/>
@@ -15984,7 +15984,7 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-12</t>
+          <t>SHARPE-11</t>
         </is>
       </c>
       <c r="C278" s="10" t="inlineStr">
@@ -15999,17 +15999,17 @@
       </c>
       <c r="E278" s="6" t="inlineStr">
         <is>
-          <t>Sharpe consistency check</t>
+          <t>Per-trade Sharpe attribution</t>
         </is>
       </c>
       <c r="F278" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
         </is>
       </c>
       <c r="G278" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
+          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr"/>
@@ -16038,7 +16038,7 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-2</t>
+          <t>SHARPE-12</t>
         </is>
       </c>
       <c r="C279" s="10" t="inlineStr">
@@ -16053,17 +16053,17 @@
       </c>
       <c r="E279" s="6" t="inlineStr">
         <is>
-          <t>Sharpe column in v2 dashboard</t>
+          <t>Sharpe consistency check</t>
         </is>
       </c>
       <c r="F279" s="5" t="inlineStr">
         <is>
-          <t>Surface 126d Sharpe per ticker as sortable column</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G279" s="5" t="inlineStr">
         <is>
-          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
+          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr"/>
@@ -16092,7 +16092,7 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-3</t>
+          <t>SHARPE-2</t>
         </is>
       </c>
       <c r="C280" s="10" t="inlineStr">
@@ -16107,17 +16107,17 @@
       </c>
       <c r="E280" s="6" t="inlineStr">
         <is>
-          <t>Per-stock Sharpe by regime</t>
+          <t>Sharpe column in v2 dashboard</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>Decompose per-stock Sharpe by historical regime tags</t>
+          <t>Surface 126d Sharpe per ticker as sortable column</t>
         </is>
       </c>
       <c r="G280" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
+          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr"/>
@@ -16146,7 +16146,7 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-4</t>
+          <t>SHARPE-3</t>
         </is>
       </c>
       <c r="C281" s="10" t="inlineStr">
@@ -16161,17 +16161,17 @@
       </c>
       <c r="E281" s="6" t="inlineStr">
         <is>
-          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
+          <t>Per-stock Sharpe by regime</t>
         </is>
       </c>
       <c r="F281" s="5" t="inlineStr">
         <is>
-          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
+          <t>Decompose per-stock Sharpe by historical regime tags</t>
         </is>
       </c>
       <c r="G281" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
+          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr"/>
@@ -16200,7 +16200,7 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-5</t>
+          <t>SHARPE-4</t>
         </is>
       </c>
       <c r="C282" s="10" t="inlineStr">
@@ -16215,17 +16215,17 @@
       </c>
       <c r="E282" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-weighted position sizing</t>
+          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
         </is>
       </c>
       <c r="G282" s="5" t="inlineStr">
         <is>
-          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr"/>
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-6</t>
+          <t>SHARPE-5</t>
         </is>
       </c>
       <c r="C283" s="10" t="inlineStr">
@@ -16269,17 +16269,17 @@
       </c>
       <c r="E283" s="6" t="inlineStr">
         <is>
-          <t>Portfolio Sharpe KPI vs target</t>
+          <t>Sharpe-weighted position sizing</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>Annualized Sharpe target tracking + gap report</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G283" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
+          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr"/>
@@ -16308,7 +16308,7 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-7</t>
+          <t>SHARPE-6</t>
         </is>
       </c>
       <c r="C284" s="10" t="inlineStr">
@@ -16323,17 +16323,17 @@
       </c>
       <c r="E284" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-based stop sizing</t>
+          <t>Portfolio Sharpe KPI vs target</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Annualized Sharpe target tracking + gap report</t>
         </is>
       </c>
       <c r="G284" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr"/>
@@ -16362,7 +16362,7 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-8</t>
+          <t>SHARPE-7</t>
         </is>
       </c>
       <c r="C285" s="10" t="inlineStr">
@@ -16377,17 +16377,17 @@
       </c>
       <c r="E285" s="6" t="inlineStr">
         <is>
-          <t>Sortino computation alongside Sharpe</t>
+          <t>Sharpe-based stop sizing</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>Downside-only vol denominator added everywhere</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G285" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
+          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr"/>
@@ -16416,7 +16416,7 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-9</t>
+          <t>SHARPE-8</t>
         </is>
       </c>
       <c r="C286" s="10" t="inlineStr">
@@ -16431,17 +16431,17 @@
       </c>
       <c r="E286" s="6" t="inlineStr">
         <is>
-          <t>SPY-Sharpe regime cross-validation</t>
+          <t>Sortino computation alongside Sharpe</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Downside-only vol denominator added everywhere</t>
         </is>
       </c>
       <c r="G286" s="5" t="inlineStr">
         <is>
-          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
+          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr"/>
@@ -16464,13 +16464,13 @@
       </c>
       <c r="N286" s="8" t="inlineStr"/>
     </row>
-    <row r="287" ht="60" customHeight="1">
+    <row r="287" ht="45" customHeight="1">
       <c r="A287" s="2" t="n">
         <v>286</v>
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-RECUR-CHIP</t>
+          <t>SHARPE-9</t>
         </is>
       </c>
       <c r="C287" s="10" t="inlineStr">
@@ -16480,22 +16480,22 @@
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>Signal Scanner</t>
+          <t>Sharpe Roadmap</t>
         </is>
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>Recurrence chip</t>
+          <t>SPY-Sharpe regime cross-validation</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G287" s="5" t="inlineStr">
         <is>
-          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr"/>
@@ -16508,23 +16508,23 @@
       </c>
       <c r="L287" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M287" s="3" t="inlineStr">
         <is>
-          <t>cf702f2b4</t>
+          <t>dbbd6b5f6</t>
         </is>
       </c>
       <c r="N287" s="8" t="inlineStr"/>
     </row>
-    <row r="288" ht="120" customHeight="1">
+    <row r="288" ht="60" customHeight="1">
       <c r="A288" s="2" t="n">
         <v>287</v>
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>CONVICTION-TIER-WIRE</t>
+          <t>SCANNER-RECUR-CHIP</t>
         </is>
       </c>
       <c r="C288" s="10" t="inlineStr">
@@ -16534,39 +16534,27 @@
       </c>
       <c r="D288" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Conviction</t>
+          <t>Signal Scanner</t>
         </is>
       </c>
       <c r="E288" s="6" t="inlineStr">
         <is>
-          <t>Conviction tier: simplified to score-band only</t>
+          <t>Recurrence chip</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
+          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
         </is>
       </c>
       <c r="G288" s="5" t="inlineStr">
         <is>
-          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
-        </is>
-      </c>
-      <c r="H288" s="2" t="inlineStr">
-        <is>
-          <t>2-4 hrs + backtest validation</t>
-        </is>
-      </c>
-      <c r="I288" s="5" t="inlineStr">
-        <is>
-          <t>Medium — changes live size or eliminates a layer</t>
-        </is>
-      </c>
-      <c r="J288" s="5" t="inlineStr">
-        <is>
-          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
-        </is>
-      </c>
+          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+        </is>
+      </c>
+      <c r="H288" s="2" t="inlineStr"/>
+      <c r="I288" s="5" t="inlineStr"/>
+      <c r="J288" s="5" t="inlineStr"/>
       <c r="K288" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16574,27 +16562,23 @@
       </c>
       <c r="L288" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M288" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N288" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
-        </is>
-      </c>
-    </row>
-    <row r="289" ht="75" customHeight="1">
+          <t>cf702f2b4</t>
+        </is>
+      </c>
+      <c r="N288" s="8" t="inlineStr"/>
+    </row>
+    <row r="289" ht="120" customHeight="1">
       <c r="A289" s="2" t="n">
         <v>288</v>
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-Q-AB</t>
+          <t>CONVICTION-TIER-WIRE</t>
         </is>
       </c>
       <c r="C289" s="10" t="inlineStr">
@@ -16604,27 +16588,39 @@
       </c>
       <c r="D289" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Gates</t>
+          <t>Strategy / Conviction</t>
         </is>
       </c>
       <c r="E289" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional entry_quality A/B</t>
+          <t>Conviction tier: simplified to score-band only</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
+          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
         </is>
       </c>
       <c r="G289" s="5" t="inlineStr">
         <is>
-          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
-        </is>
-      </c>
-      <c r="H289" s="2" t="inlineStr"/>
-      <c r="I289" s="5" t="inlineStr"/>
-      <c r="J289" s="5" t="inlineStr"/>
+          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr">
+        <is>
+          <t>2-4 hrs + backtest validation</t>
+        </is>
+      </c>
+      <c r="I289" s="5" t="inlineStr">
+        <is>
+          <t>Medium — changes live size or eliminates a layer</t>
+        </is>
+      </c>
+      <c r="J289" s="5" t="inlineStr">
+        <is>
+          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
+        </is>
+      </c>
       <c r="K289" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16632,23 +16628,27 @@
       </c>
       <c r="L289" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M289" s="3" t="inlineStr">
         <is>
-          <t>07c3af6a3</t>
-        </is>
-      </c>
-      <c r="N289" s="8" t="inlineStr"/>
-    </row>
-    <row r="290" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N289" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
+        </is>
+      </c>
+    </row>
+    <row r="290" ht="75" customHeight="1">
       <c r="A290" s="2" t="n">
         <v>289</v>
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-1</t>
+          <t>ENTRY-Q-AB</t>
         </is>
       </c>
       <c r="C290" s="10" t="inlineStr">
@@ -16658,22 +16658,22 @@
       </c>
       <c r="D290" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Options Paper</t>
+          <t>Strategy / Gates</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
         <is>
-          <t>Signal -&gt; options-structure mapper</t>
+          <t>Regime-conditional entry_quality A/B</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
         <is>
-          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
+          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
         </is>
       </c>
       <c r="G290" s="5" t="inlineStr">
         <is>
-          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
+          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
         </is>
       </c>
       <c r="H290" s="2" t="inlineStr"/>
@@ -16686,23 +16686,23 @@
       </c>
       <c r="L290" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr">
         <is>
-          <t>9c3a2a58d</t>
+          <t>07c3af6a3</t>
         </is>
       </c>
       <c r="N290" s="8" t="inlineStr"/>
     </row>
-    <row r="291" ht="45" customHeight="1">
+    <row r="291" ht="60" customHeight="1">
       <c r="A291" s="2" t="n">
         <v>290</v>
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-2</t>
+          <t>OPT-PAPER-1</t>
         </is>
       </c>
       <c r="C291" s="10" t="inlineStr">
@@ -16717,17 +16717,17 @@
       </c>
       <c r="E291" s="6" t="inlineStr">
         <is>
-          <t>Contract selection from Schwab chain</t>
+          <t>Signal -&gt; options-structure mapper</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
+          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
         </is>
       </c>
       <c r="G291" s="5" t="inlineStr">
         <is>
-          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
+          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr"/>
@@ -16750,13 +16750,13 @@
       </c>
       <c r="N291" s="8" t="inlineStr"/>
     </row>
-    <row r="292" ht="60" customHeight="1">
+    <row r="292" ht="45" customHeight="1">
       <c r="A292" s="2" t="n">
         <v>291</v>
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-3</t>
+          <t>OPT-PAPER-2</t>
         </is>
       </c>
       <c r="C292" s="10" t="inlineStr">
@@ -16771,17 +16771,17 @@
       </c>
       <c r="E292" s="6" t="inlineStr">
         <is>
-          <t>Alpaca paper options orders in executor.py</t>
+          <t>Contract selection from Schwab chain</t>
         </is>
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
+          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
         </is>
       </c>
       <c r="G292" s="5" t="inlineStr">
         <is>
-          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
+          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr"/>
@@ -16804,13 +16804,13 @@
       </c>
       <c r="N292" s="8" t="inlineStr"/>
     </row>
-    <row r="293" ht="45" customHeight="1">
+    <row r="293" ht="60" customHeight="1">
       <c r="A293" s="2" t="n">
         <v>292</v>
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-4</t>
+          <t>OPT-PAPER-3</t>
         </is>
       </c>
       <c r="C293" s="10" t="inlineStr">
@@ -16825,17 +16825,17 @@
       </c>
       <c r="E293" s="6" t="inlineStr">
         <is>
-          <t>Options position tracking + contract P&amp;L</t>
+          <t>Alpaca paper options orders in executor.py</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
+          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
         </is>
       </c>
       <c r="G293" s="5" t="inlineStr">
         <is>
-          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
+          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
         </is>
       </c>
       <c r="H293" s="2" t="inlineStr"/>
@@ -16853,7 +16853,7 @@
       </c>
       <c r="M293" s="3" t="inlineStr">
         <is>
-          <t>635ae960f</t>
+          <t>9c3a2a58d</t>
         </is>
       </c>
       <c r="N293" s="8" t="inlineStr"/>
@@ -16864,7 +16864,7 @@
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-5</t>
+          <t>OPT-PAPER-4</t>
         </is>
       </c>
       <c r="C294" s="10" t="inlineStr">
@@ -16879,17 +16879,17 @@
       </c>
       <c r="E294" s="6" t="inlineStr">
         <is>
-          <t>Options-specific exits</t>
+          <t>Options position tracking + contract P&amp;L</t>
         </is>
       </c>
       <c r="F294" s="5" t="inlineStr">
         <is>
-          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
+          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
         </is>
       </c>
       <c r="G294" s="5" t="inlineStr">
         <is>
-          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
+          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr"/>
@@ -16912,13 +16912,13 @@
       </c>
       <c r="N294" s="8" t="inlineStr"/>
     </row>
-    <row r="295" ht="120" customHeight="1">
+    <row r="295" ht="45" customHeight="1">
       <c r="A295" s="2" t="n">
         <v>294</v>
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>UI-STRAT-1</t>
+          <t>OPT-PAPER-5</t>
         </is>
       </c>
       <c r="C295" s="10" t="inlineStr">
@@ -16928,22 +16928,22 @@
       </c>
       <c r="D295" s="5" t="inlineStr">
         <is>
-          <t>Strategy Lab</t>
+          <t>Strategy / Options Paper</t>
         </is>
       </c>
       <c r="E295" s="6" t="inlineStr">
         <is>
-          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
+          <t>Options-specific exits</t>
         </is>
       </c>
       <c r="F295" s="5" t="inlineStr">
         <is>
-          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
+          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
         </is>
       </c>
       <c r="G295" s="5" t="inlineStr">
         <is>
-          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
+          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
         </is>
       </c>
       <c r="H295" s="2" t="inlineStr"/>
@@ -16956,23 +16956,23 @@
       </c>
       <c r="L295" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="M295" s="3" t="inlineStr">
         <is>
-          <t>93ec11842</t>
+          <t>635ae960f</t>
         </is>
       </c>
       <c r="N295" s="8" t="inlineStr"/>
     </row>
-    <row r="296" ht="60" customHeight="1">
+    <row r="296" ht="120" customHeight="1">
       <c r="A296" s="2" t="n">
         <v>295</v>
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>TE-SESSION-CACHE</t>
+          <t>UI-STRAT-1</t>
         </is>
       </c>
       <c r="C296" s="10" t="inlineStr">
@@ -16982,22 +16982,22 @@
       </c>
       <c r="D296" s="5" t="inlineStr">
         <is>
-          <t>Structural Targets</t>
+          <t>Strategy Lab</t>
         </is>
       </c>
       <c r="E296" s="6" t="inlineStr">
         <is>
-          <t>Session-date cache invalidation</t>
+          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
         </is>
       </c>
       <c r="F296" s="5" t="inlineStr">
         <is>
-          <t>target_engine cache used 12h wall-clock TTL → expired mid-session (15:00-19:30 PT dead-zone) causing on-demand recomputes on tab open</t>
+          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
         </is>
       </c>
       <c r="G296" s="5" t="inlineStr">
         <is>
-          <t>Switched _cache_is_fresh to session-date keying (_latest_completed_session) + 36h backstop + legacy grandfather; _cache_write stamps session_date. 0 added EODHD, recompute only on new daily bar.</t>
+          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr"/>
@@ -17010,12 +17010,12 @@
       </c>
       <c r="L296" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr">
         <is>
-          <t>33146be5e</t>
+          <t>93ec11842</t>
         </is>
       </c>
       <c r="N296" s="8" t="inlineStr"/>
@@ -17026,7 +17026,7 @@
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>TE-STRATEGY-MODE</t>
+          <t>TE-SESSION-CACHE</t>
         </is>
       </c>
       <c r="C297" s="10" t="inlineStr">
@@ -17036,22 +17036,22 @@
       </c>
       <c r="D297" s="5" t="inlineStr">
         <is>
-          <t>Target Engine</t>
+          <t>Structural Targets</t>
         </is>
       </c>
       <c r="E297" s="6" t="inlineStr">
         <is>
-          <t>_strategy_mode read but never written</t>
+          <t>Session-date cache invalidation</t>
         </is>
       </c>
       <c r="F297" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
+          <t>target_engine cache used 12h wall-clock TTL → expired mid-session (15:00-19:30 PT dead-zone) causing on-demand recomputes on tab open</t>
         </is>
       </c>
       <c r="G297" s="5" t="inlineStr">
         <is>
-          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
+          <t>Switched _cache_is_fresh to session-date keying (_latest_completed_session) + 36h backstop + legacy grandfather; _cache_write stamps session_date. 0 added EODHD, recompute only on new daily bar.</t>
         </is>
       </c>
       <c r="H297" s="2" t="inlineStr"/>
@@ -17064,23 +17064,23 @@
       </c>
       <c r="L297" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>33146be5e</t>
         </is>
       </c>
       <c r="N297" s="8" t="inlineStr"/>
     </row>
-    <row r="298" ht="105" customHeight="1">
+    <row r="298" ht="60" customHeight="1">
       <c r="A298" s="2" t="n">
         <v>297</v>
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>TRACKER-BUY-FILTER</t>
+          <t>TE-STRATEGY-MODE</t>
         </is>
       </c>
       <c r="C298" s="10" t="inlineStr">
@@ -17090,31 +17090,27 @@
       </c>
       <c r="D298" s="5" t="inlineStr">
         <is>
-          <t>Tracker/Feedback Loop</t>
+          <t>Target Engine</t>
         </is>
       </c>
       <c r="E298" s="6" t="inlineStr">
         <is>
-          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
+          <t>_strategy_mode read but never written</t>
         </is>
       </c>
       <c r="F298" s="5" t="inlineStr">
         <is>
-          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
+          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
         </is>
       </c>
       <c r="G298" s="5" t="inlineStr">
         <is>
-          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
         </is>
       </c>
       <c r="H298" s="2" t="inlineStr"/>
       <c r="I298" s="5" t="inlineStr"/>
-      <c r="J298" s="5" t="inlineStr">
-        <is>
-          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
-        </is>
-      </c>
+      <c r="J298" s="5" t="inlineStr"/>
       <c r="K298" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17122,27 +17118,23 @@
       </c>
       <c r="L298" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M298" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N298" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="299" ht="135" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N298" s="8" t="inlineStr"/>
+    </row>
+    <row r="299" ht="105" customHeight="1">
       <c r="A299" s="2" t="n">
         <v>298</v>
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
+          <t>TRACKER-BUY-FILTER</t>
         </is>
       </c>
       <c r="C299" s="10" t="inlineStr">
@@ -17152,37 +17144,29 @@
       </c>
       <c r="D299" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Tracker/Feedback Loop</t>
         </is>
       </c>
       <c r="E299" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
         </is>
       </c>
       <c r="F299" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
         </is>
       </c>
       <c r="G299" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
-        </is>
-      </c>
-      <c r="H299" s="2" t="inlineStr">
-        <is>
-          <t>1-2 hrs</t>
-        </is>
-      </c>
-      <c r="I299" s="5" t="inlineStr">
-        <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
-        </is>
-      </c>
+          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+        </is>
+      </c>
+      <c r="H299" s="2" t="inlineStr"/>
+      <c r="I299" s="5" t="inlineStr"/>
       <c r="J299" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
         </is>
       </c>
       <c r="K299" s="12" t="inlineStr">
@@ -17192,27 +17176,27 @@
       </c>
       <c r="L299" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M299" s="3" t="inlineStr">
         <is>
-          <t>42c36ef91</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N299" s="8" t="inlineStr">
         <is>
-          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="300" ht="45" customHeight="1">
+          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="300" ht="135" customHeight="1">
       <c r="A300" s="2" t="n">
         <v>299</v>
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>STOCKSMITH-BOOK-RISK</t>
+          <t>MOD-1</t>
         </is>
       </c>
       <c r="C300" s="10" t="inlineStr">
@@ -17222,27 +17206,39 @@
       </c>
       <c r="D300" s="5" t="inlineStr">
         <is>
-          <t>V2 Dashboard / Risk</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E300" s="6" t="inlineStr">
         <is>
-          <t>Book Risk surface + per-lens analytics (§6)</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F300" s="5" t="inlineStr">
         <is>
-          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G300" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
-        </is>
-      </c>
-      <c r="H300" s="2" t="inlineStr"/>
-      <c r="I300" s="5" t="inlineStr"/>
-      <c r="J300" s="5" t="inlineStr"/>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I300" s="5" t="inlineStr">
+        <is>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
+        </is>
+      </c>
+      <c r="J300" s="5" t="inlineStr">
+        <is>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+        </is>
+      </c>
       <c r="K300" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17250,23 +17246,27 @@
       </c>
       <c r="L300" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr">
         <is>
-          <t>50cace567</t>
-        </is>
-      </c>
-      <c r="N300" s="8" t="inlineStr"/>
-    </row>
-    <row r="301" ht="120" customHeight="1">
+          <t>42c36ef91</t>
+        </is>
+      </c>
+      <c r="N300" s="8" t="inlineStr">
+        <is>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="45" customHeight="1">
       <c r="A301" s="2" t="n">
         <v>300</v>
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>RECENCY-FLOOR</t>
+          <t>STOCKSMITH-BOOK-RISK</t>
         </is>
       </c>
       <c r="C301" s="10" t="inlineStr">
@@ -17276,31 +17276,27 @@
       </c>
       <c r="D301" s="5" t="inlineStr">
         <is>
-          <t>Validation Hygiene</t>
+          <t>V2 Dashboard / Risk</t>
         </is>
       </c>
       <c r="E301" s="6" t="inlineStr">
         <is>
-          <t>_validations needs recency floor — auto-revert stale boosts</t>
+          <t>Book Risk surface + per-lens analytics (§6)</t>
         </is>
       </c>
       <c r="F301" s="5" t="inlineStr">
         <is>
-          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
+          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
         </is>
       </c>
       <c r="G301" s="5" t="inlineStr">
         <is>
-          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
+          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
         </is>
       </c>
       <c r="H301" s="2" t="inlineStr"/>
       <c r="I301" s="5" t="inlineStr"/>
-      <c r="J301" s="5" t="inlineStr">
-        <is>
-          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
-        </is>
-      </c>
+      <c r="J301" s="5" t="inlineStr"/>
       <c r="K301" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17308,27 +17304,23 @@
       </c>
       <c r="L301" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N301" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="302" ht="60" customHeight="1">
+          <t>50cace567</t>
+        </is>
+      </c>
+      <c r="N301" s="8" t="inlineStr"/>
+    </row>
+    <row r="302" ht="120" customHeight="1">
       <c r="A302" s="2" t="n">
         <v>301</v>
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-TAB</t>
+          <t>RECENCY-FLOOR</t>
         </is>
       </c>
       <c r="C302" s="10" t="inlineStr">
@@ -17338,27 +17330,31 @@
       </c>
       <c r="D302" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Momentum</t>
+          <t>Validation Hygiene</t>
         </is>
       </c>
       <c r="E302" s="6" t="inlineStr">
         <is>
-          <t>New 🚀 Momentum workspace tab</t>
+          <t>_validations needs recency floor — auto-revert stale boosts</t>
         </is>
       </c>
       <c r="F302" s="5" t="inlineStr">
         <is>
-          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
+          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
         </is>
       </c>
       <c r="G302" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
+          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
         </is>
       </c>
       <c r="H302" s="2" t="inlineStr"/>
       <c r="I302" s="5" t="inlineStr"/>
-      <c r="J302" s="5" t="inlineStr"/>
+      <c r="J302" s="5" t="inlineStr">
+        <is>
+          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
+        </is>
+      </c>
       <c r="K302" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17366,15 +17362,19 @@
       </c>
       <c r="L302" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N302" s="8" t="inlineStr"/>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N302" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
+        </is>
+      </c>
     </row>
     <row r="303" ht="60" customHeight="1">
       <c r="A303" s="2" t="n">
@@ -17382,7 +17382,7 @@
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-QUICK-PANELS</t>
+          <t>MOMENTUM-TAB</t>
         </is>
       </c>
       <c r="C303" s="10" t="inlineStr">
@@ -17392,22 +17392,22 @@
       </c>
       <c r="D303" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Signal Scanner</t>
+          <t>Workspaces / Momentum</t>
         </is>
       </c>
       <c r="E303" s="6" t="inlineStr">
         <is>
-          <t>5 quick-glance panels above watchlist table</t>
+          <t>New 🚀 Momentum workspace tab</t>
         </is>
       </c>
       <c r="F303" s="5" t="inlineStr">
         <is>
-          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
+          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
         </is>
       </c>
       <c r="G303" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
         </is>
       </c>
       <c r="H303" s="2" t="inlineStr"/>
@@ -17425,60 +17425,48 @@
       </c>
       <c r="M303" s="3" t="inlineStr">
         <is>
-          <t>dfbe955fe</t>
+          <t>27fd646b1</t>
         </is>
       </c>
       <c r="N303" s="8" t="inlineStr"/>
     </row>
-    <row r="304" ht="45" customHeight="1">
+    <row r="304" ht="60" customHeight="1">
       <c r="A304" s="2" t="n">
         <v>303</v>
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C304" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>SCANNER-QUICK-PANELS</t>
+        </is>
+      </c>
+      <c r="C304" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D304" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Workspaces / Signal Scanner</t>
         </is>
       </c>
       <c r="E304" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>5 quick-glance panels above watchlist table</t>
         </is>
       </c>
       <c r="F304" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
         </is>
       </c>
       <c r="G304" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
-        </is>
-      </c>
-      <c r="H304" s="2" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="I304" s="5" t="inlineStr">
-        <is>
-          <t>Win: persistence works; no silent overwrites.</t>
-        </is>
-      </c>
-      <c r="J304" s="5" t="inlineStr">
-        <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
-        </is>
-      </c>
+          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+        </is>
+      </c>
+      <c r="H304" s="2" t="inlineStr"/>
+      <c r="I304" s="5" t="inlineStr"/>
+      <c r="J304" s="5" t="inlineStr"/>
       <c r="K304" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17486,15 +17474,15 @@
       </c>
       <c r="L304" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M304" s="3" t="inlineStr"/>
-      <c r="N304" s="8" t="inlineStr">
-        <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="M304" s="3" t="inlineStr">
+        <is>
+          <t>dfbe955fe</t>
+        </is>
+      </c>
+      <c r="N304" s="8" t="inlineStr"/>
     </row>
     <row r="305" ht="45" customHeight="1">
       <c r="A305" s="2" t="n">
@@ -17502,7 +17490,7 @@
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="C305" s="13" t="inlineStr">
@@ -17517,32 +17505,32 @@
       </c>
       <c r="E305" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F305" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G305" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H305" s="2" t="inlineStr">
         <is>
-          <t>verified (no change needed)</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I305" s="5" t="inlineStr">
         <is>
-          <t>Win: confirms infrastructure still healthy.</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J305" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
         </is>
       </c>
       <c r="K305" s="12" t="inlineStr">
@@ -17558,7 +17546,7 @@
       <c r="M305" s="3" t="inlineStr"/>
       <c r="N305" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
         </is>
       </c>
     </row>
@@ -17568,7 +17556,7 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>UI-3</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -17578,35 +17566,39 @@
       </c>
       <c r="D306" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E306" s="6" t="inlineStr">
         <is>
-          <t>Remove emoji icons from Thesis + Research labels</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F306" s="5" t="inlineStr">
         <is>
-          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G306" s="5" t="inlineStr">
         <is>
-          <t>Removed emojis from FD sub-tab nav + section headers.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H306" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I306" s="5" t="inlineStr">
         <is>
-          <t>Low / cosmetic</t>
-        </is>
-      </c>
-      <c r="J306" s="5" t="inlineStr"/>
+          <t>Win: confirms infrastructure still healthy.</t>
+        </is>
+      </c>
+      <c r="J306" s="5" t="inlineStr">
+        <is>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
       <c r="K306" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17614,17 +17606,13 @@
       </c>
       <c r="L306" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="M306" s="3" t="inlineStr">
-        <is>
-          <t>24fd7c273</t>
-        </is>
-      </c>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M306" s="3" t="inlineStr"/>
       <c r="N306" s="8" t="inlineStr">
         <is>
-          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
         </is>
       </c>
     </row>
@@ -17634,59 +17622,63 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
-        </is>
-      </c>
-      <c r="C307" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>UI-3</t>
+        </is>
+      </c>
+      <c r="C307" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D307" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E307" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Remove emoji icons from Thesis + Research labels</t>
         </is>
       </c>
       <c r="F307" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
         </is>
       </c>
       <c r="G307" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+          <t>Removed emojis from FD sub-tab nav + section headers.</t>
         </is>
       </c>
       <c r="H307" s="2" t="inlineStr">
         <is>
-          <t>5 min after answer</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I307" s="5" t="inlineStr">
         <is>
-          <t>Win: -671 lines.</t>
-        </is>
-      </c>
-      <c r="J307" s="5" t="inlineStr">
-        <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K307" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L307" s="2" t="inlineStr"/>
-      <c r="M307" s="3" t="inlineStr"/>
+          <t>Low / cosmetic</t>
+        </is>
+      </c>
+      <c r="J307" s="5" t="inlineStr"/>
+      <c r="K307" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L307" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M307" s="3" t="inlineStr">
+        <is>
+          <t>24fd7c273</t>
+        </is>
+      </c>
       <c r="N307" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
         </is>
       </c>
     </row>
@@ -17696,7 +17688,7 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
+          <t>CLEAN-2</t>
         </is>
       </c>
       <c r="C308" s="10" t="inlineStr">
@@ -17706,37 +17698,37 @@
       </c>
       <c r="D308" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E308" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
         </is>
       </c>
       <c r="F308" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
         </is>
       </c>
       <c r="G308" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
         </is>
       </c>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>5 min after answer</t>
         </is>
       </c>
       <c r="I308" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Win: -671 lines.</t>
         </is>
       </c>
       <c r="J308" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
+          <t>Standard data-migration retention practice.</t>
         </is>
       </c>
       <c r="K308" s="14" t="inlineStr">
@@ -17758,109 +17750,109 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C309" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C309" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D309" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E309" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
         </is>
       </c>
       <c r="F309" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
         </is>
       </c>
       <c r="G309" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
         </is>
       </c>
       <c r="H309" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>hours-days each</t>
         </is>
       </c>
       <c r="I309" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win varies; defer until PERF-7 measured.</t>
         </is>
       </c>
       <c r="J309" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K309" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K309" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="L309" s="2" t="inlineStr"/>
       <c r="M309" s="3" t="inlineStr"/>
       <c r="N309" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="310" ht="75" customHeight="1">
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="310" ht="45" customHeight="1">
       <c r="A310" s="2" t="n">
         <v>309</v>
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>MOD-2</t>
-        </is>
-      </c>
-      <c r="C310" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C310" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D310" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E310" s="6" t="inlineStr">
         <is>
-          <t>Pixel-diff regression baseline</t>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
         </is>
       </c>
       <c r="F310" s="5" t="inlineStr">
         <is>
-          <t>After modularization, no automated visual-regression catch.</t>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
         </is>
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
         </is>
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I310" s="5" t="inlineStr">
         <is>
-          <t>Win: catches accidental layout regressions.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J310" s="5" t="inlineStr">
         <is>
-          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+          <t>Agents skim and miss post-filter subset analysis.</t>
         </is>
       </c>
       <c r="K310" s="15" t="inlineStr">
@@ -17868,147 +17860,209 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L310" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
+      <c r="L310" s="2" t="inlineStr"/>
       <c r="M310" s="3" t="inlineStr"/>
       <c r="N310" s="8" t="inlineStr">
         <is>
-          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="311" ht="195" customHeight="1">
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="75" customHeight="1">
       <c r="A311" s="2" t="n">
         <v>310</v>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
+          <t>MOD-2</t>
+        </is>
+      </c>
+      <c r="C311" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D311" s="5" t="inlineStr">
+        <is>
+          <t>UI / Modularization</t>
+        </is>
+      </c>
+      <c r="E311" s="6" t="inlineStr">
+        <is>
+          <t>Pixel-diff regression baseline</t>
+        </is>
+      </c>
+      <c r="F311" s="5" t="inlineStr">
+        <is>
+          <t>After modularization, no automated visual-regression catch.</t>
+        </is>
+      </c>
+      <c r="G311" s="5" t="inlineStr">
+        <is>
+          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+        </is>
+      </c>
+      <c r="H311" s="2" t="inlineStr">
+        <is>
+          <t>2-3 hrs</t>
+        </is>
+      </c>
+      <c r="I311" s="5" t="inlineStr">
+        <is>
+          <t>Win: catches accidental layout regressions.</t>
+        </is>
+      </c>
+      <c r="J311" s="5" t="inlineStr">
+        <is>
+          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+        </is>
+      </c>
+      <c r="K311" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L311" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="M311" s="3" t="inlineStr"/>
+      <c r="N311" s="8" t="inlineStr">
+        <is>
+          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="195" customHeight="1">
+      <c r="A312" s="2" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
           <t>OB-CONFLUENCE-PROPOSAL-REJECTED</t>
         </is>
       </c>
-      <c r="C311" s="10" t="inlineStr">
+      <c r="C312" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D311" s="5" t="inlineStr">
+      <c r="D312" s="5" t="inlineStr">
         <is>
           <t>Signals / Cross-Check</t>
         </is>
       </c>
-      <c r="E311" s="6" t="inlineStr">
+      <c r="E312" s="6" t="inlineStr">
         <is>
           <t>OB-confluence Wilson bump + OB-aware stop — proposals KILLED by backtest evidence</t>
         </is>
       </c>
-      <c r="F311" s="5" t="inlineStr">
+      <c r="F312" s="5" t="inlineStr">
         <is>
           <t>User asked 2026-05-12 to ship #2 (Wilson-bump score factor for bullish OB confluence within 5% of entry) and #5 (OB-low as stop instead of 1.25xATR). Per Principle 1 / Principle 7, ran post-hoc validation: scripts/validate_ob_confluence.py retroactively tags every closed trade from existing portfolio_backtest outputs with SMC state at entry date, computes Wilson 95% LB per subset.
 RESULT (750-day backtest · n=384): Bull OB confluence within 5% of entry DECREASES Wilson LB by -8.6pp (14.6% vs baseline 23.1%). BOS-bullish boost: -3.4pp. SMC-bullish direction boost: -3.6pp. Per #5 simulation, 35 of 39 (90%) OB-low-as-stop would have loosened the stop; 25 of those still ended in losses (looser stops do not rescue broken setups, they extend exposure).
 Principle 4 fires: proposals FALSIFIED, killed permanently (not retuned). Doing the change without this validation would have introduced a 6-9pp Wilson-LB drag on every BUY signal.</t>
         </is>
       </c>
-      <c r="G311" s="5" t="inlineStr">
+      <c r="G312" s="5" t="inlineStr">
         <is>
           <t>Built scripts/validate_ob_confluence.py to retroactively run smart_money.score_smc() on the historical OHLCV at each trade's entry date, tag with OB-confluence + BOS + CHoCH flags, compute Wilson 95% LB per subset, and apply Principle 1 gates (n&gt;=30, lift&gt;=5pp). Cross-validated on 250d (n=142) and 750d (n=384) backtest outputs. Both agree: NO EDGE.</t>
         </is>
       </c>
-      <c r="H311" s="2" t="inlineStr">
+      <c r="H312" s="2" t="inlineStr">
         <is>
           <t>Days of work avoided (would have shipped a degrading change).</t>
         </is>
       </c>
-      <c r="I311" s="5" t="inlineStr">
+      <c r="I312" s="5" t="inlineStr">
         <is>
           <t>Mechanism (Principle 2): institutional OBs are supposed to mark re-add zones for smart money. Falsification (Principle 4): if the data doesn't show OB-confluent trades winning more, the mechanism either doesn't exist for retail-accessible OB detection at daily resolution OR is already priced into our 5-pillar score. Either way: ship nothing. The proposals are dead. Win: prevented a 6-9pp Wilson-LB drag from being added to live scoring. Lost: nothing — we didn't change live scoring, no opportunity cost.</t>
         </is>
       </c>
-      <c r="J311" s="5" t="inlineStr">
+      <c r="J312" s="5" t="inlineStr">
         <is>
           <t>Validator script is reusable infrastructure. Re-run any time the SMC detection logic or score thresholds change. NOTE: baseline WR in 750d backtest is 27.3% (low) — the absolute level reflects backtest-window-specific market conditions; the SUBSET comparisons are valid regardless because they share the same baseline. Do not interpret 23.1% Wilson LB as a system-level edge — that's a separate question. This validation answers ONLY: does OB-confluence improve selection within whatever the system already does.</t>
         </is>
       </c>
-      <c r="K311" s="15" t="inlineStr">
+      <c r="K312" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L311" s="2" t="inlineStr">
+      <c r="L312" s="2" t="inlineStr">
         <is>
           <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="M311" s="3" t="inlineStr"/>
-      <c r="N311" s="8" t="inlineStr">
-        <is>
-          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="312" ht="90" customHeight="1">
-      <c r="A312" s="2" t="n">
-        <v>311</v>
-      </c>
-      <c r="B312" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C312" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="D312" s="5" t="inlineStr">
-        <is>
-          <t>Data / Universe</t>
-        </is>
-      </c>
-      <c r="E312" s="6" t="inlineStr">
-        <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
-        </is>
-      </c>
-      <c r="F312" s="5" t="inlineStr">
-        <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
-        </is>
-      </c>
-      <c r="G312" s="5" t="inlineStr">
-        <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
-        </is>
-      </c>
-      <c r="H312" s="2" t="inlineStr">
-        <is>
-          <t>$$ + 1 day</t>
-        </is>
-      </c>
-      <c r="I312" s="5" t="inlineStr">
-        <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
-        </is>
-      </c>
-      <c r="J312" s="5" t="inlineStr">
-        <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K312" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L312" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M312" s="3" t="inlineStr"/>
       <c r="N312" s="8" t="inlineStr">
+        <is>
+          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="90" customHeight="1">
+      <c r="A313" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C313" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D313" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E313" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F313" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G313" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H313" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I313" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J313" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K313" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L313" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M313" s="3" t="inlineStr"/>
+      <c r="N313" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -18113,10 +18167,10 @@
         <v>90</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="5">
@@ -18170,10 +18224,10 @@
         <v>115</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FEAT: code backup to NAS (git-mirror + rsync) (NAS-CODE-BACKUP)
Off-Mac code backup to the Synology CodeBackup SMB share, two channels each using
the right tool:
- A) git push --mirror to a bare repo on the NAS (/volume1/CodeBackup/SwingTrade.git)
  — efficient packed transfer of all branches+history, vs rsync crawling thousands
  of loose .git objects over SMB.
- B) rsync of working files (excl .git/cache/node_modules + the SMB-reserved names
  CON/PRN/AUX/NUL that the protocol can't create — hit data/ohlcv/CON.parquet).

Verified by test-cloning the NAS mirror: valid repo, 731 commits, 4948 files, all
3 branches. Nightly via com.swingtrade.code-backup (21:00 PT, LaunchAgent so the
SMB mount is visible). Restore: git clone /Volumes/CodeBackup/SwingTrade.git

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-06-18.xlsx
+++ b/cache/open_items_2026-06-18.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N313"/>
+  <dimension ref="A1:N314"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -14854,7 +14854,7 @@
       </c>
       <c r="B259" s="3" t="inlineStr">
         <is>
-          <t>NAS-HISTORY-SYNC</t>
+          <t>NAS-CODE-BACKUP</t>
         </is>
       </c>
       <c r="C259" s="10" t="inlineStr">
@@ -14869,17 +14869,17 @@
       </c>
       <c r="E259" s="6" t="inlineStr">
         <is>
-          <t>Sync all track-history to NAS deep store</t>
+          <t>Code backup to NAS CodeBackup share</t>
         </is>
       </c>
       <c r="F259" s="5" t="inlineStr">
         <is>
-          <t>Only ticker_snapshots was on NAS; signal_log/audit_ledger/picks_history/ml_edge existed only locally — not a true backup</t>
+          <t>Needed an off-Mac code backup before cleaning the 89%-full disk; rsync-over-SMB crawled on .git loose objects</t>
         </is>
       </c>
       <c r="G259" s="5" t="inlineStr">
         <is>
-          <t>nas_pg.archive_json (JSONB archive, NaN-sanitized, in-batch dedup); scripts/sync_history_to_nas.py mirrors signal_log(4713)/audit_ledger(4915)/picks_trades(1766)/picks_runs(57)/ml_edge(1905); nightly via scripts/nas_sync_all.sh in com.swingtrade.nas-sync; 209,630 total rows on NAS</t>
+          <t>scripts/backup_code_to_nas.sh: (A) git push --mirror to bare repo on NAS (efficient packed transfer, all branches), (B) rsync working files excl .git/cache/node_modules + SMB reserved names (CON/PRN/AUX/NUL). Verified via test-clone: 731 commits/4948 files. Nightly com.swingtrade.code-backup 21:00 PT</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr"/>
@@ -14897,18 +14897,18 @@
       </c>
       <c r="M259" s="3" t="inlineStr">
         <is>
-          <t>cb4ef7114</t>
+          <t>4c2deb164</t>
         </is>
       </c>
       <c r="N259" s="8" t="inlineStr"/>
     </row>
-    <row r="260" ht="90" customHeight="1">
+    <row r="260" ht="75" customHeight="1">
       <c r="A260" s="2" t="n">
         <v>259</v>
       </c>
       <c r="B260" s="3" t="inlineStr">
         <is>
-          <t>NAS-PG-DEEP-STORE</t>
+          <t>NAS-HISTORY-SYNC</t>
         </is>
       </c>
       <c r="C260" s="10" t="inlineStr">
@@ -14923,17 +14923,17 @@
       </c>
       <c r="E260" s="6" t="inlineStr">
         <is>
-          <t>Self-hosted Postgres on Synology NAS as deep audit/snapshot store</t>
+          <t>Sync all track-history to NAS deep store</t>
         </is>
       </c>
       <c r="F260" s="5" t="inlineStr">
         <is>
-          <t>Local SQLite limited by 162GB-free disk (89% full); full snapshot retention untenable locally. Owner has DS1520+ NAS</t>
+          <t>Only ticker_snapshots was on NAS; signal_log/audit_ledger/picks_history/ml_edge existed only locally — not a true backup</t>
         </is>
       </c>
       <c r="G260" s="5" t="inlineStr">
         <is>
-          <t>Postgres 16 container on DS1520+ (192.168.1.25:5433); nas_pg.py (conn+schema+upsert), scripts/sync_snapshots_to_nas.py (idempotent push), ticker_snapshots.capture_scan best-effort real-time push, nightly catch-up launchd com.swingtrade.nas-sync. SQLite=hot 90d, NAS=full retention. 196K rows synced, raw_gz round-trips 292 fields. NAS_PG_URL in .env (gitignored)</t>
+          <t>nas_pg.archive_json (JSONB archive, NaN-sanitized, in-batch dedup); scripts/sync_history_to_nas.py mirrors signal_log(4713)/audit_ledger(4915)/picks_trades(1766)/picks_runs(57)/ml_edge(1905); nightly via scripts/nas_sync_all.sh in com.swingtrade.nas-sync; 209,630 total rows on NAS</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr"/>
@@ -14951,7 +14951,7 @@
       </c>
       <c r="M260" s="3" t="inlineStr">
         <is>
-          <t>76cca4dbd</t>
+          <t>cb4ef7114</t>
         </is>
       </c>
       <c r="N260" s="8" t="inlineStr"/>
@@ -14962,7 +14962,7 @@
       </c>
       <c r="B261" s="3" t="inlineStr">
         <is>
-          <t>UI-MLEDGE-1</t>
+          <t>NAS-PG-DEEP-STORE</t>
         </is>
       </c>
       <c r="C261" s="10" t="inlineStr">
@@ -14972,22 +14972,22 @@
       </c>
       <c r="D261" s="5" t="inlineStr">
         <is>
-          <t>ML Edge Tab</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E261" s="6" t="inlineStr">
         <is>
-          <t>Theme switching + tf-* visual port</t>
+          <t>Self-hosted Postgres on Synology NAS as deep audit/snapshot store</t>
         </is>
       </c>
       <c r="F261" s="5" t="inlineStr">
         <is>
-          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
+          <t>Local SQLite limited by 162GB-free disk (89% full); full snapshot retention untenable locally. Owner has DS1520+ NAS</t>
         </is>
       </c>
       <c r="G261" s="5" t="inlineStr">
         <is>
-          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
+          <t>Postgres 16 container on DS1520+ (192.168.1.25:5433); nas_pg.py (conn+schema+upsert), scripts/sync_snapshots_to_nas.py (idempotent push), ticker_snapshots.capture_scan best-effort real-time push, nightly catch-up launchd com.swingtrade.nas-sync. SQLite=hot 90d, NAS=full retention. 196K rows synced, raw_gz round-trips 292 fields. NAS_PG_URL in .env (gitignored)</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr"/>
@@ -15000,23 +15000,23 @@
       </c>
       <c r="L261" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="M261" s="3" t="inlineStr">
         <is>
-          <t>696731a4d</t>
+          <t>76cca4dbd</t>
         </is>
       </c>
       <c r="N261" s="8" t="inlineStr"/>
     </row>
-    <row r="262" ht="45" customHeight="1">
+    <row r="262" ht="90" customHeight="1">
       <c r="A262" s="2" t="n">
         <v>261</v>
       </c>
       <c r="B262" s="3" t="inlineStr">
         <is>
-          <t>IPAD-2</t>
+          <t>UI-MLEDGE-1</t>
         </is>
       </c>
       <c r="C262" s="10" t="inlineStr">
@@ -15026,39 +15026,27 @@
       </c>
       <c r="D262" s="5" t="inlineStr">
         <is>
-          <t>Mobile / iPad</t>
+          <t>ML Edge Tab</t>
         </is>
       </c>
       <c r="E262" s="6" t="inlineStr">
         <is>
-          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
+          <t>Theme switching + tf-* visual port</t>
         </is>
       </c>
       <c r="F262" s="5" t="inlineStr">
         <is>
-          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
+          <t>ML Edge per-ticker sub-tab had hardcoded dark CSS vars inline on #qd-ml-root, blocking the body.light theme toggle. Workspace ML Edge used legacy rk-* class system, not the prototype tf-* design language.</t>
         </is>
       </c>
       <c r="G262" s="5" t="inlineStr">
         <is>
-          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
-        </is>
-      </c>
-      <c r="H262" s="2" t="inlineStr">
-        <is>
-          <t>15 min</t>
-        </is>
-      </c>
-      <c r="I262" s="5" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="J262" s="5" t="inlineStr">
-        <is>
-          <t>Sub-task of IPAD-1.</t>
-        </is>
-      </c>
+          <t>Moved palette from inline style to _ensureMlEdgeStyles() with body.light overrides. Then ported workspace QuantMlEdge module to tf-* visual system: tf-hero 3-col + tf-pulse-strip 4 live feeds (top bulls/bears/flips/health) + tf-confluence (4 KPI cells + X/4 score) + tf-vbar (verdict badge). All 6 sections rewritten. Memory: feedback_inline_css_vars_break_theming.md.</t>
+        </is>
+      </c>
+      <c r="H262" s="2" t="inlineStr"/>
+      <c r="I262" s="5" t="inlineStr"/>
+      <c r="J262" s="5" t="inlineStr"/>
       <c r="K262" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15066,19 +15054,15 @@
       </c>
       <c r="L262" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M262" s="3" t="inlineStr">
         <is>
-          <t>79fa01a75</t>
-        </is>
-      </c>
-      <c r="N262" s="8" t="inlineStr">
-        <is>
-          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
-        </is>
-      </c>
+          <t>696731a4d</t>
+        </is>
+      </c>
+      <c r="N262" s="8" t="inlineStr"/>
     </row>
     <row r="263" ht="45" customHeight="1">
       <c r="A263" s="2" t="n">
@@ -15086,7 +15070,7 @@
       </c>
       <c r="B263" s="3" t="inlineStr">
         <is>
-          <t>SLACK-NEWSLETTER-MLALERT</t>
+          <t>IPAD-2</t>
         </is>
       </c>
       <c r="C263" s="10" t="inlineStr">
@@ -15096,27 +15080,39 @@
       </c>
       <c r="D263" s="5" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Mobile / iPad</t>
         </is>
       </c>
       <c r="E263" s="6" t="inlineStr">
         <is>
-          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
+          <t>elite-detail iframe-embed mode (hide FLOOR sidebar)</t>
         </is>
       </c>
       <c r="F263" s="5" t="inlineStr">
         <is>
-          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
+          <t>Detail iframe inside iPad shell wasted 80px width on FLOOR sidebar.</t>
         </is>
       </c>
       <c r="G263" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd + scripts/ml_alert_slack.py</t>
-        </is>
-      </c>
-      <c r="H263" s="2" t="inlineStr"/>
-      <c r="I263" s="5" t="inlineStr"/>
-      <c r="J263" s="5" t="inlineStr"/>
+          <t>Detect iframe context (window.parent !== window) and hide floor.css elements.</t>
+        </is>
+      </c>
+      <c r="H263" s="2" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="I263" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="J263" s="5" t="inlineStr">
+        <is>
+          <t>Sub-task of IPAD-1.</t>
+        </is>
+      </c>
       <c r="K263" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15124,15 +15120,19 @@
       </c>
       <c r="L263" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M263" s="3" t="inlineStr">
         <is>
-          <t>d1ea97913</t>
-        </is>
-      </c>
-      <c r="N263" s="8" t="inlineStr"/>
+          <t>79fa01a75</t>
+        </is>
+      </c>
+      <c r="N263" s="8" t="inlineStr">
+        <is>
+          <t>Open iPad shell, tap a ticker → detail iframe should NOT show FLOOR left sidebar.</t>
+        </is>
+      </c>
     </row>
     <row r="264" ht="45" customHeight="1">
       <c r="A264" s="2" t="n">
@@ -15140,7 +15140,7 @@
       </c>
       <c r="B264" s="3" t="inlineStr">
         <is>
-          <t>FORENSICS-WEEKLY-SLACK</t>
+          <t>SLACK-NEWSLETTER-MLALERT</t>
         </is>
       </c>
       <c r="C264" s="10" t="inlineStr">
@@ -15150,22 +15150,22 @@
       </c>
       <c r="D264" s="5" t="inlineStr">
         <is>
-          <t>Notifications / Audit</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="E264" s="6" t="inlineStr">
         <is>
-          <t>Weekly pick-forensics Slack digest</t>
+          <t>Re-enable newsletter + add ML-predictions Slack alert</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
         <is>
-          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
+          <t>re-enable daily-newsletter from disabled/; build ml-alert Slack for top ML-edge/AI picks</t>
         </is>
       </c>
       <c r="G264" s="5" t="inlineStr">
         <is>
-          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+          <t>infra/launchd + scripts/ml_alert_slack.py</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr"/>
@@ -15183,18 +15183,18 @@
       </c>
       <c r="M264" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>d1ea97913</t>
         </is>
       </c>
       <c r="N264" s="8" t="inlineStr"/>
     </row>
-    <row r="265" ht="75" customHeight="1">
+    <row r="265" ht="45" customHeight="1">
       <c r="A265" s="2" t="n">
         <v>264</v>
       </c>
       <c r="B265" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
+          <t>FORENSICS-WEEKLY-SLACK</t>
         </is>
       </c>
       <c r="C265" s="10" t="inlineStr">
@@ -15204,39 +15204,27 @@
       </c>
       <c r="D265" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Notifications / Audit</t>
         </is>
       </c>
       <c r="E265" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Weekly pick-forensics Slack digest</t>
         </is>
       </c>
       <c r="F265" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>Sun 17:30 — 14d verdict-truth + per-sleeve EXTENDED/MISSED bleeding monitor to Slack</t>
         </is>
       </c>
       <c r="G265" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
-        </is>
-      </c>
-      <c r="H265" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I265" s="5" t="inlineStr">
-        <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
-        </is>
-      </c>
-      <c r="J265" s="5" t="inlineStr">
-        <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
-        </is>
-      </c>
+          <t>com.swingtrade.forensics-weekly + pick_forensics --slack</t>
+        </is>
+      </c>
+      <c r="H265" s="2" t="inlineStr"/>
+      <c r="I265" s="5" t="inlineStr"/>
+      <c r="J265" s="5" t="inlineStr"/>
       <c r="K265" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15244,27 +15232,23 @@
       </c>
       <c r="L265" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M265" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
-        </is>
-      </c>
-      <c r="N265" s="8" t="inlineStr">
-        <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="266" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N265" s="8" t="inlineStr"/>
+    </row>
+    <row r="266" ht="75" customHeight="1">
       <c r="A266" s="2" t="n">
         <v>265</v>
       </c>
       <c r="B266" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C266" s="10" t="inlineStr">
@@ -15274,37 +15258,37 @@
       </c>
       <c r="D266" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E266" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F266" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G266" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I266" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J266" s="5" t="inlineStr">
         <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K266" s="12" t="inlineStr">
@@ -15314,17 +15298,17 @@
       </c>
       <c r="L266" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M266" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N266" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
         </is>
       </c>
     </row>
@@ -15334,7 +15318,7 @@
       </c>
       <c r="B267" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C267" s="10" t="inlineStr">
@@ -15349,32 +15333,32 @@
       </c>
       <c r="E267" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F267" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G267" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I267" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J267" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K267" s="12" t="inlineStr">
@@ -15394,7 +15378,7 @@
       </c>
       <c r="N267" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -15404,7 +15388,7 @@
       </c>
       <c r="B268" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C268" s="10" t="inlineStr">
@@ -15419,32 +15403,32 @@
       </c>
       <c r="E268" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F268" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G268" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I268" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J268" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K268" s="12" t="inlineStr">
@@ -15464,7 +15448,7 @@
       </c>
       <c r="N268" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
         </is>
       </c>
     </row>
@@ -15474,7 +15458,7 @@
       </c>
       <c r="B269" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>OPS-4</t>
         </is>
       </c>
       <c r="C269" s="10" t="inlineStr">
@@ -15489,32 +15473,32 @@
       </c>
       <c r="E269" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F269" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G269" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H269" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I269" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J269" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K269" s="12" t="inlineStr">
@@ -15524,27 +15508,27 @@
       </c>
       <c r="L269" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M269" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N269" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="270" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="270" ht="60" customHeight="1">
       <c r="A270" s="2" t="n">
         <v>269</v>
       </c>
       <c r="B270" s="3" t="inlineStr">
         <is>
-          <t>SCAN-FAILURE-ALERT</t>
+          <t>OPS-5</t>
         </is>
       </c>
       <c r="C270" s="10" t="inlineStr">
@@ -15554,27 +15538,39 @@
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>Ops / Alerts</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E270" s="6" t="inlineStr">
         <is>
-          <t>Scan-failure + EODHD-quota Slack alert</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F270" s="5" t="inlineStr">
         <is>
-          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G270" s="5" t="inlineStr">
         <is>
-          <t>swing_trade.py exit hook</t>
-        </is>
-      </c>
-      <c r="H270" s="2" t="inlineStr"/>
-      <c r="I270" s="5" t="inlineStr"/>
-      <c r="J270" s="5" t="inlineStr"/>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+        </is>
+      </c>
+      <c r="H270" s="2" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="I270" s="5" t="inlineStr">
+        <is>
+          <t>Win: fast iteration on report templates.</t>
+        </is>
+      </c>
+      <c r="J270" s="5" t="inlineStr">
+        <is>
+          <t>Trivial CLI wrapper.</t>
+        </is>
+      </c>
       <c r="K270" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15582,15 +15578,19 @@
       </c>
       <c r="L270" s="2" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M270" s="3" t="inlineStr">
         <is>
-          <t>0dc7675ee</t>
-        </is>
-      </c>
-      <c r="N270" s="8" t="inlineStr"/>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N270" s="8" t="inlineStr">
+        <is>
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
     </row>
     <row r="271" ht="45" customHeight="1">
       <c r="A271" s="2" t="n">
@@ -15598,7 +15598,7 @@
       </c>
       <c r="B271" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
+          <t>SCAN-FAILURE-ALERT</t>
         </is>
       </c>
       <c r="C271" s="10" t="inlineStr">
@@ -15608,22 +15608,22 @@
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>Ops / Launchd</t>
+          <t>Ops / Alerts</t>
         </is>
       </c>
       <c r="E271" s="6" t="inlineStr">
         <is>
-          <t>Decide momentum-snapshot: load or retire</t>
+          <t>Scan-failure + EODHD-quota Slack alert</t>
         </is>
       </c>
       <c r="F271" s="5" t="inlineStr">
         <is>
-          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
+          <t>failed scan / 402 quota is silent today; 1-line health alert on scan exit</t>
         </is>
       </c>
       <c r="G271" s="5" t="inlineStr">
         <is>
-          <t>infra/launchd</t>
+          <t>swing_trade.py exit hook</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr"/>
@@ -15646,13 +15646,13 @@
       </c>
       <c r="N271" s="8" t="inlineStr"/>
     </row>
-    <row r="272" ht="60" customHeight="1">
+    <row r="272" ht="45" customHeight="1">
       <c r="A272" s="2" t="n">
         <v>271</v>
       </c>
       <c r="B272" s="3" t="inlineStr">
         <is>
-          <t>OVERVIEW-TQ-LABEL</t>
+          <t>MOMENTUM-SNAPSHOT-DECIDE</t>
         </is>
       </c>
       <c r="C272" s="10" t="inlineStr">
@@ -15662,22 +15662,22 @@
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>Overview</t>
+          <t>Ops / Launchd</t>
         </is>
       </c>
       <c r="E272" s="6" t="inlineStr">
         <is>
-          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
+          <t>Decide momentum-snapshot: load or retire</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
         <is>
-          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
+          <t>valid plist, not loaded; PARSE-ERR on lint earlier</t>
         </is>
       </c>
       <c r="G272" s="5" t="inlineStr">
         <is>
-          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
+          <t>infra/launchd</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr"/>
@@ -15690,23 +15690,23 @@
       </c>
       <c r="L272" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-31</t>
         </is>
       </c>
       <c r="M272" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>0dc7675ee</t>
         </is>
       </c>
       <c r="N272" s="8" t="inlineStr"/>
     </row>
-    <row r="273" ht="150" customHeight="1">
+    <row r="273" ht="60" customHeight="1">
       <c r="A273" s="2" t="n">
         <v>272</v>
       </c>
       <c r="B273" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>OVERVIEW-TQ-LABEL</t>
         </is>
       </c>
       <c r="C273" s="10" t="inlineStr">
@@ -15716,31 +15716,27 @@
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Overview</t>
         </is>
       </c>
       <c r="E273" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Strategy-Fit verdict used action verbs colliding with canonical verdict</t>
         </is>
       </c>
       <c r="F273" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>_deriveVerdict emitted BUY·ENTER/HOLD·ADD DIP/WEAK·SKIP from target-quality math in same vocabulary as canonical BUY/WATCH/AVOID action verdict — user could misread the target-quality chip as THE verdict</t>
         </is>
       </c>
       <c r="G273" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+          <t>relabel to PRIME/GOOD/WEAK TARGET nouns under a TARGET QUALITY caption; canonical exec-brief verdict (binds T.stage) untouched</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr"/>
       <c r="I273" s="5" t="inlineStr"/>
-      <c r="J273" s="5" t="inlineStr">
-        <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
-        </is>
-      </c>
+      <c r="J273" s="5" t="inlineStr"/>
       <c r="K273" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15748,27 +15744,23 @@
       </c>
       <c r="L273" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M273" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
-        </is>
-      </c>
-      <c r="N273" s="8" t="inlineStr">
-        <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="274" ht="105" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N273" s="8" t="inlineStr"/>
+    </row>
+    <row r="274" ht="150" customHeight="1">
       <c r="A274" s="2" t="n">
         <v>273</v>
       </c>
       <c r="B274" s="3" t="inlineStr">
         <is>
-          <t>SMC-OB-DISPLAY-1</t>
+          <t>PERF-7b</t>
         </is>
       </c>
       <c r="C274" s="10" t="inlineStr">
@@ -15778,27 +15770,31 @@
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>SMC</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E274" s="6" t="inlineStr">
         <is>
-          <t>OB confluence badges in SMC tab</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F274" s="5" t="inlineStr">
         <is>
-          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G274" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr"/>
       <c r="I274" s="5" t="inlineStr"/>
-      <c r="J274" s="5" t="inlineStr"/>
+      <c r="J274" s="5" t="inlineStr">
+        <is>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+        </is>
+      </c>
       <c r="K274" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -15806,23 +15802,27 @@
       </c>
       <c r="L274" s="2" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M274" s="3" t="inlineStr">
         <is>
-          <t>8182c3977</t>
-        </is>
-      </c>
-      <c r="N274" s="8" t="inlineStr"/>
-    </row>
-    <row r="275" ht="75" customHeight="1">
+          <t>cf30df858</t>
+        </is>
+      </c>
+      <c r="N274" s="8" t="inlineStr">
+        <is>
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="275" ht="105" customHeight="1">
       <c r="A275" s="2" t="n">
         <v>274</v>
       </c>
       <c r="B275" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-COMPANY-NAMES</t>
+          <t>SMC-OB-DISPLAY-1</t>
         </is>
       </c>
       <c r="C275" s="10" t="inlineStr">
@@ -15832,22 +15832,22 @@
       </c>
       <c r="D275" s="5" t="inlineStr">
         <is>
-          <t>Scanner UI</t>
+          <t>SMC</t>
         </is>
       </c>
       <c r="E275" s="6" t="inlineStr">
         <is>
-          <t>NAME column duplicated TICKER (no company names)</t>
+          <t>OB confluence badges in SMC tab</t>
         </is>
       </c>
       <c r="F275" s="5" t="inlineStr">
         <is>
-          <t>Scan feed set name=ticker; no cached name source (fundamentals.db raw_json has 0 names). NAME column was redundant.</t>
+          <t>SMC-tab order blocks (engines/smc.py) showed bare lo/hi/type/state — no BOS/FVG/volume/HTF/reaction confluence context for the user to judge OB quality.</t>
         </is>
       </c>
       <c r="G275" s="5" t="inlineStr">
         <is>
-          <t>Free Wikipedia S&amp;P1500+NDX+Dow name map (scripts/build_ticker_names.py -&gt; cache/ticker_names.json, 1508 names); joined in /api/universe _ticker_names(); weekly refresh in weekly_diagnostics.sh. 70% live coverage, honest ticker fallback for the tail. No paid data.</t>
+          <t>Phase 1 (display-only, informational): engines/smc.py._order_blocks + detect() enrich each OB with bos_type/rel_vol/has_fvg/htf_aligned/reaction/confluence[]/confluence_n; surfaced as a Confluence column + chips in lens-smc-risk.jsx and a board tag in surface-smc-patterns.jsx. smc_score + ranking UNCHANGED. Phase 2 (re-rank on these factors) deferred until OB Wilson-bucket win-rates clear n&gt;=30 OOS per the 500-user signal-enable bar.</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr"/>
@@ -15860,23 +15860,23 @@
       </c>
       <c r="L275" s="2" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="M275" s="3" t="inlineStr">
         <is>
-          <t>48f6a2fbf</t>
+          <t>8182c3977</t>
         </is>
       </c>
       <c r="N275" s="8" t="inlineStr"/>
     </row>
-    <row r="276" ht="45" customHeight="1">
+    <row r="276" ht="75" customHeight="1">
       <c r="A276" s="2" t="n">
         <v>275</v>
       </c>
       <c r="B276" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-1</t>
+          <t>SCANNER-COMPANY-NAMES</t>
         </is>
       </c>
       <c r="C276" s="10" t="inlineStr">
@@ -15886,22 +15886,22 @@
       </c>
       <c r="D276" s="5" t="inlineStr">
         <is>
-          <t>Sharpe Roadmap</t>
+          <t>Scanner UI</t>
         </is>
       </c>
       <c r="E276" s="6" t="inlineStr">
         <is>
-          <t>Sharpe gate in momentum detector</t>
+          <t>NAME column duplicated TICKER (no company names)</t>
         </is>
       </c>
       <c r="F276" s="5" t="inlineStr">
         <is>
-          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
+          <t>Scan feed set name=ticker; no cached name source (fundamentals.db raw_json has 0 names). NAME column was redundant.</t>
         </is>
       </c>
       <c r="G276" s="5" t="inlineStr">
         <is>
-          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
+          <t>Free Wikipedia S&amp;P1500+NDX+Dow name map (scripts/build_ticker_names.py -&gt; cache/ticker_names.json, 1508 names); joined in /api/universe _ticker_names(); weekly refresh in weekly_diagnostics.sh. 70% live coverage, honest ticker fallback for the tail. No paid data.</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr"/>
@@ -15914,12 +15914,12 @@
       </c>
       <c r="L276" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="M276" s="3" t="inlineStr">
         <is>
-          <t>dbbd6b5f6</t>
+          <t>48f6a2fbf</t>
         </is>
       </c>
       <c r="N276" s="8" t="inlineStr"/>
@@ -15930,7 +15930,7 @@
       </c>
       <c r="B277" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-10</t>
+          <t>SHARPE-1</t>
         </is>
       </c>
       <c r="C277" s="10" t="inlineStr">
@@ -15945,17 +15945,17 @@
       </c>
       <c r="E277" s="6" t="inlineStr">
         <is>
-          <t>Sharpe alerts for watchlist</t>
+          <t>Sharpe gate in momentum detector</t>
         </is>
       </c>
       <c r="F277" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Wire 126d Sharpe threshold (≥1.5) into _detect_momentum_continuation</t>
         </is>
       </c>
       <c r="G277" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
+          <t>Computed inline in analyze_ticker via lib.sharpe_utils.sharpe_annualized; passed to detector as kwarg</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr"/>
@@ -15984,7 +15984,7 @@
       </c>
       <c r="B278" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-11</t>
+          <t>SHARPE-10</t>
         </is>
       </c>
       <c r="C278" s="10" t="inlineStr">
@@ -15999,17 +15999,17 @@
       </c>
       <c r="E278" s="6" t="inlineStr">
         <is>
-          <t>Per-trade Sharpe attribution</t>
+          <t>Sharpe alerts for watchlist</t>
         </is>
       </c>
       <c r="F278" s="5" t="inlineStr">
         <is>
-          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G278" s="5" t="inlineStr">
         <is>
-          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
+          <t>scripts/sharpe_alert.py — tracks state across runs, posts to SLACK_WEBHOOK_URL</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr"/>
@@ -16038,7 +16038,7 @@
       </c>
       <c r="B279" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-12</t>
+          <t>SHARPE-11</t>
         </is>
       </c>
       <c r="C279" s="10" t="inlineStr">
@@ -16053,17 +16053,17 @@
       </c>
       <c r="E279" s="6" t="inlineStr">
         <is>
-          <t>Sharpe consistency check</t>
+          <t>Per-trade Sharpe attribution</t>
         </is>
       </c>
       <c r="F279" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Decompose portfolio Sharpe by ticker / setup / regime contribution</t>
         </is>
       </c>
       <c r="G279" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
+          <t>Built into scripts/sharpe_kpi.py — top contributors / detractors + setup + regime contribution tables</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr"/>
@@ -16092,7 +16092,7 @@
       </c>
       <c r="B280" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-2</t>
+          <t>SHARPE-12</t>
         </is>
       </c>
       <c r="C280" s="10" t="inlineStr">
@@ -16107,17 +16107,17 @@
       </c>
       <c r="E280" s="6" t="inlineStr">
         <is>
-          <t>Sharpe column in v2 dashboard</t>
+          <t>Sharpe consistency check</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>Surface 126d Sharpe per ticker as sortable column</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G280" s="5" t="inlineStr">
         <is>
-          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
+          <t>lib.sharpe_utils.rolling_sharpe + consistency_score; surfaced on per-ticker result dict</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr"/>
@@ -16146,7 +16146,7 @@
       </c>
       <c r="B281" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-3</t>
+          <t>SHARPE-2</t>
         </is>
       </c>
       <c r="C281" s="10" t="inlineStr">
@@ -16161,17 +16161,17 @@
       </c>
       <c r="E281" s="6" t="inlineStr">
         <is>
-          <t>Per-stock Sharpe by regime</t>
+          <t>Sharpe column in v2 dashboard</t>
         </is>
       </c>
       <c r="F281" s="5" t="inlineStr">
         <is>
-          <t>Decompose per-stock Sharpe by historical regime tags</t>
+          <t>Surface 126d Sharpe per ticker as sortable column</t>
         </is>
       </c>
       <c r="G281" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
+          <t>Added sharpe_126d / sortino_126d / sharpe_consistency to compact_row in build_data.py</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr"/>
@@ -16200,7 +16200,7 @@
       </c>
       <c r="B282" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-4</t>
+          <t>SHARPE-3</t>
         </is>
       </c>
       <c r="C282" s="10" t="inlineStr">
@@ -16215,17 +16215,17 @@
       </c>
       <c r="E282" s="6" t="inlineStr">
         <is>
-          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
+          <t>Per-stock Sharpe by regime</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
+          <t>Decompose per-stock Sharpe by historical regime tags</t>
         </is>
       </c>
       <c r="G282" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
+          <t>scripts/sharpe_per_regime.py — segments OHLCV by regime, computes per-bucket Sharpe</t>
         </is>
       </c>
       <c r="H282" s="2" t="inlineStr"/>
@@ -16254,7 +16254,7 @@
       </c>
       <c r="B283" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-5</t>
+          <t>SHARPE-4</t>
         </is>
       </c>
       <c r="C283" s="10" t="inlineStr">
@@ -16269,17 +16269,17 @@
       </c>
       <c r="E283" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-weighted position sizing</t>
+          <t>Edge-erosion radar (per-setup Sharpe trend)</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Per-setup Sharpe across rolling windows w/ HTML viz</t>
         </is>
       </c>
       <c r="G283" s="5" t="inlineStr">
         <is>
-          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_setup_trend.py — emits trend table + dark-themed HTML chart per setup</t>
         </is>
       </c>
       <c r="H283" s="2" t="inlineStr"/>
@@ -16308,7 +16308,7 @@
       </c>
       <c r="B284" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-6</t>
+          <t>SHARPE-5</t>
         </is>
       </c>
       <c r="C284" s="10" t="inlineStr">
@@ -16323,17 +16323,17 @@
       </c>
       <c r="E284" s="6" t="inlineStr">
         <is>
-          <t>Portfolio Sharpe KPI vs target</t>
+          <t>Sharpe-weighted position sizing</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>Annualized Sharpe target tracking + gap report</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G284" s="5" t="inlineStr">
         <is>
-          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
+          <t>kelly_position_size new sharpe_126d kwarg + portfolio.sharpe_size_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H284" s="2" t="inlineStr"/>
@@ -16362,7 +16362,7 @@
       </c>
       <c r="B285" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-7</t>
+          <t>SHARPE-6</t>
         </is>
       </c>
       <c r="C285" s="10" t="inlineStr">
@@ -16377,17 +16377,17 @@
       </c>
       <c r="E285" s="6" t="inlineStr">
         <is>
-          <t>Sharpe-based stop sizing</t>
+          <t>Portfolio Sharpe KPI vs target</t>
         </is>
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Annualized Sharpe target tracking + gap report</t>
         </is>
       </c>
       <c r="G285" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
+          <t>scripts/sharpe_kpi.py — reports actual vs target/floor, exits 2 on below-floor for cron alerts</t>
         </is>
       </c>
       <c r="H285" s="2" t="inlineStr"/>
@@ -16416,7 +16416,7 @@
       </c>
       <c r="B286" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-8</t>
+          <t>SHARPE-7</t>
         </is>
       </c>
       <c r="C286" s="10" t="inlineStr">
@@ -16431,17 +16431,17 @@
       </c>
       <c r="E286" s="6" t="inlineStr">
         <is>
-          <t>Sortino computation alongside Sharpe</t>
+          <t>Sharpe-based stop sizing</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>Downside-only vol denominator added everywhere</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G286" s="5" t="inlineStr">
         <is>
-          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
+          <t>compute_trade_plan reads runtime sharpe; portfolio.sharpe_stop_tilt config block (default OFF)</t>
         </is>
       </c>
       <c r="H286" s="2" t="inlineStr"/>
@@ -16470,7 +16470,7 @@
       </c>
       <c r="B287" s="3" t="inlineStr">
         <is>
-          <t>SHARPE-9</t>
+          <t>SHARPE-8</t>
         </is>
       </c>
       <c r="C287" s="10" t="inlineStr">
@@ -16485,17 +16485,17 @@
       </c>
       <c r="E287" s="6" t="inlineStr">
         <is>
-          <t>SPY-Sharpe regime cross-validation</t>
+          <t>Sortino computation alongside Sharpe</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>Implements item from Sharpe roadmap brainstorm</t>
+          <t>Downside-only vol denominator added everywhere</t>
         </is>
       </c>
       <c r="G287" s="5" t="inlineStr">
         <is>
-          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
+          <t>lib.sharpe_utils.sortino_annualized + per_trade_sortino; surfaced on result dict</t>
         </is>
       </c>
       <c r="H287" s="2" t="inlineStr"/>
@@ -16518,13 +16518,13 @@
       </c>
       <c r="N287" s="8" t="inlineStr"/>
     </row>
-    <row r="288" ht="60" customHeight="1">
+    <row r="288" ht="45" customHeight="1">
       <c r="A288" s="2" t="n">
         <v>287</v>
       </c>
       <c r="B288" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-RECUR-CHIP</t>
+          <t>SHARPE-9</t>
         </is>
       </c>
       <c r="C288" s="10" t="inlineStr">
@@ -16534,22 +16534,22 @@
       </c>
       <c r="D288" s="5" t="inlineStr">
         <is>
-          <t>Signal Scanner</t>
+          <t>Sharpe Roadmap</t>
         </is>
       </c>
       <c r="E288" s="6" t="inlineStr">
         <is>
-          <t>Recurrence chip</t>
+          <t>SPY-Sharpe regime cross-validation</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
+          <t>Implements item from Sharpe roadmap brainstorm</t>
         </is>
       </c>
       <c r="G288" s="5" t="inlineStr">
         <is>
-          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+          <t>data_fetcher.get_market_regime now includes spy_sharpe payload</t>
         </is>
       </c>
       <c r="H288" s="2" t="inlineStr"/>
@@ -16562,23 +16562,23 @@
       </c>
       <c r="L288" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M288" s="3" t="inlineStr">
         <is>
-          <t>cf702f2b4</t>
+          <t>dbbd6b5f6</t>
         </is>
       </c>
       <c r="N288" s="8" t="inlineStr"/>
     </row>
-    <row r="289" ht="120" customHeight="1">
+    <row r="289" ht="60" customHeight="1">
       <c r="A289" s="2" t="n">
         <v>288</v>
       </c>
       <c r="B289" s="3" t="inlineStr">
         <is>
-          <t>CONVICTION-TIER-WIRE</t>
+          <t>SCANNER-RECUR-CHIP</t>
         </is>
       </c>
       <c r="C289" s="10" t="inlineStr">
@@ -16588,39 +16588,27 @@
       </c>
       <c r="D289" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Conviction</t>
+          <t>Signal Scanner</t>
         </is>
       </c>
       <c r="E289" s="6" t="inlineStr">
         <is>
-          <t>Conviction tier: simplified to score-band only</t>
+          <t>Recurrence chip</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
+          <t>Per-ticker 'seen N× + W-L' chip on scanner rows, deep-links to Track Record · The Ledger filtered for that ticker</t>
         </is>
       </c>
       <c r="G289" s="5" t="inlineStr">
         <is>
-          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
-        </is>
-      </c>
-      <c r="H289" s="2" t="inlineStr">
-        <is>
-          <t>2-4 hrs + backtest validation</t>
-        </is>
-      </c>
-      <c r="I289" s="5" t="inlineStr">
-        <is>
-          <t>Medium — changes live size or eliminates a layer</t>
-        </is>
-      </c>
-      <c r="J289" s="5" t="inlineStr">
-        <is>
-          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
-        </is>
-      </c>
+          <t>Server: _signal_recurrence_map() over signal_log.json joined onto /api/universe; boot maps recurrence→seen/wlb/n/pf; SeenChip in surface-signal.jsx; window.__trkIntent one-shot intent consumed by SurfaceTrackRecord</t>
+        </is>
+      </c>
+      <c r="H289" s="2" t="inlineStr"/>
+      <c r="I289" s="5" t="inlineStr"/>
+      <c r="J289" s="5" t="inlineStr"/>
       <c r="K289" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16628,27 +16616,23 @@
       </c>
       <c r="L289" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M289" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N289" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
-        </is>
-      </c>
-    </row>
-    <row r="290" ht="75" customHeight="1">
+          <t>cf702f2b4</t>
+        </is>
+      </c>
+      <c r="N289" s="8" t="inlineStr"/>
+    </row>
+    <row r="290" ht="120" customHeight="1">
       <c r="A290" s="2" t="n">
         <v>289</v>
       </c>
       <c r="B290" s="3" t="inlineStr">
         <is>
-          <t>ENTRY-Q-AB</t>
+          <t>CONVICTION-TIER-WIRE</t>
         </is>
       </c>
       <c r="C290" s="10" t="inlineStr">
@@ -16658,27 +16642,39 @@
       </c>
       <c r="D290" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Gates</t>
+          <t>Strategy / Conviction</t>
         </is>
       </c>
       <c r="E290" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional entry_quality A/B</t>
+          <t>Conviction tier: simplified to score-band only</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
         <is>
-          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
+          <t>n=423 closed signal audit (2026-05-11): 93% of production BUYs have no conviction_label set. T1 has never fired. T2 has never fired. The tier system assigns labels via assign_conviction_tier but the live engine does not gate trades by conviction tier (size_mult or label). The ~395 unlabeled BUYs perform fine (WR 60.8%, avg +3.87%) because the OTHER filters do the work.</t>
         </is>
       </c>
       <c r="G290" s="5" t="inlineStr">
         <is>
-          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
-        </is>
-      </c>
-      <c r="H290" s="2" t="inlineStr"/>
-      <c r="I290" s="5" t="inlineStr"/>
-      <c r="J290" s="5" t="inlineStr"/>
+          <t>Option A: wire tier.size_mult into kelly_position_size as a hard scale factor. Block BUYs with tier=WATCH/AVOID. Verifies via backtest. Option B: delete the tier system; replace with simpler score-based size scaling. Either way, current state is misleading.</t>
+        </is>
+      </c>
+      <c r="H290" s="2" t="inlineStr">
+        <is>
+          <t>2-4 hrs + backtest validation</t>
+        </is>
+      </c>
+      <c r="I290" s="5" t="inlineStr">
+        <is>
+          <t>Medium — changes live size or eliminates a layer</t>
+        </is>
+      </c>
+      <c r="J290" s="5" t="inlineStr">
+        <is>
+          <t>Resolved 2026-05-11 by SIMPLIFYING (not deleting). The complex tier criteria (AND of score+RR+RS+regime+catalyst+entry_quality) had 0 T1/T2 trades ever fire in 423 closed signals. The intersection was empty — system was decorative. Replaced with score-only band: T1 score&gt;=88, T2 score&gt;=78, T3 score&gt;=70, WATCH 60-69, AVOID &lt;60. Win-rate setup adjustment retained (single-factor, evidence-driven). All callers preserved — they now get real tier labels instead of mostly-empty results.</t>
+        </is>
+      </c>
       <c r="K290" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -16686,23 +16682,27 @@
       </c>
       <c r="L290" s="2" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M290" s="3" t="inlineStr">
         <is>
-          <t>07c3af6a3</t>
-        </is>
-      </c>
-      <c r="N290" s="8" t="inlineStr"/>
-    </row>
-    <row r="291" ht="60" customHeight="1">
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N290" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import assign_conviction_tier; print([assign_conviction_tier(s)["label"] for s in [95,87,75,65,55]])' → ['T1','T2','T3','WATCH','AVOID']</t>
+        </is>
+      </c>
+    </row>
+    <row r="291" ht="75" customHeight="1">
       <c r="A291" s="2" t="n">
         <v>290</v>
       </c>
       <c r="B291" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-1</t>
+          <t>ENTRY-Q-AB</t>
         </is>
       </c>
       <c r="C291" s="10" t="inlineStr">
@@ -16712,22 +16712,22 @@
       </c>
       <c r="D291" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Options Paper</t>
+          <t>Strategy / Gates</t>
         </is>
       </c>
       <c r="E291" s="6" t="inlineStr">
         <is>
-          <t>Signal -&gt; options-structure mapper</t>
+          <t>Regime-conditional entry_quality A/B</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
+          <t>Test relaxing entry_quality EXTENDED/MISSED to caveat-only in risk_on_choppy regime. Evidence (n=257 EXTENDED PF 1.63, n=179 MISSED PF 2.89 in choppy) suggests gate is upside-down for that regime, but selection bias + market-cycle asymmetry concerns warrant explicit A/B before promoting to default.</t>
         </is>
       </c>
       <c r="G291" s="5" t="inlineStr">
         <is>
-          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
+          <t>Add config flag regime4_thresholds.risk_on_choppy.entry_quality_caveat_only (default false). Modify decision_engine to honor it. Run 30 days control + 30 days test. Compare WR/PF stratified by entry_quality band. Promote if test PF &gt; control by &gt;=0.3 with n&gt;=30 per band.</t>
         </is>
       </c>
       <c r="H291" s="2" t="inlineStr"/>
@@ -16740,23 +16740,23 @@
       </c>
       <c r="L291" s="2" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="M291" s="3" t="inlineStr">
         <is>
-          <t>9c3a2a58d</t>
+          <t>07c3af6a3</t>
         </is>
       </c>
       <c r="N291" s="8" t="inlineStr"/>
     </row>
-    <row r="292" ht="45" customHeight="1">
+    <row r="292" ht="60" customHeight="1">
       <c r="A292" s="2" t="n">
         <v>291</v>
       </c>
       <c r="B292" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-2</t>
+          <t>OPT-PAPER-1</t>
         </is>
       </c>
       <c r="C292" s="10" t="inlineStr">
@@ -16771,17 +16771,17 @@
       </c>
       <c r="E292" s="6" t="inlineStr">
         <is>
-          <t>Contract selection from Schwab chain</t>
+          <t>Signal -&gt; options-structure mapper</t>
         </is>
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
+          <t>Engine emits equity plans only; no layer maps a stock BUY to a defined-risk options structure. GATED: equity sleeves still Phase-1. See docs/scope_options_paper.md.</t>
         </is>
       </c>
       <c r="G292" s="5" t="inlineStr">
         <is>
-          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
+          <t>Map equity plan -&gt; defined-risk structure by setup family / R:R / IV rank (3:1 high-conviction -&gt; debit call spread; clean trend -&gt; long call 30-45 DTE). Underlying stop = thesis invalidation. Defined-risk ONLY, paper ONLY.</t>
         </is>
       </c>
       <c r="H292" s="2" t="inlineStr"/>
@@ -16804,13 +16804,13 @@
       </c>
       <c r="N292" s="8" t="inlineStr"/>
     </row>
-    <row r="293" ht="60" customHeight="1">
+    <row r="293" ht="45" customHeight="1">
       <c r="A293" s="2" t="n">
         <v>292</v>
       </c>
       <c r="B293" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-3</t>
+          <t>OPT-PAPER-2</t>
         </is>
       </c>
       <c r="C293" s="10" t="inlineStr">
@@ -16825,17 +16825,17 @@
       </c>
       <c r="E293" s="6" t="inlineStr">
         <is>
-          <t>Alpaca paper options orders in executor.py</t>
+          <t>Contract selection from Schwab chain</t>
         </is>
       </c>
       <c r="F293" s="5" t="inlineStr">
         <is>
-          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
+          <t>We have chain+Greeks data (schwab_client.get_chains/extract_chain_greeks) but no contract picker. Dep: SCHWAB-REAUTH-PENDING (Greeks freshness).</t>
         </is>
       </c>
       <c r="G293" s="5" t="inlineStr">
         <is>
-          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
+          <t>Pick by delta/DTE/spread width from the Schwab chain; size on premium-at-risk &lt;=1% equity. No naked options.</t>
         </is>
       </c>
       <c r="H293" s="2" t="inlineStr"/>
@@ -16858,13 +16858,13 @@
       </c>
       <c r="N293" s="8" t="inlineStr"/>
     </row>
-    <row r="294" ht="45" customHeight="1">
+    <row r="294" ht="60" customHeight="1">
       <c r="A294" s="2" t="n">
         <v>293</v>
       </c>
       <c r="B294" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-4</t>
+          <t>OPT-PAPER-3</t>
         </is>
       </c>
       <c r="C294" s="10" t="inlineStr">
@@ -16879,17 +16879,17 @@
       </c>
       <c r="E294" s="6" t="inlineStr">
         <is>
-          <t>Options position tracking + contract P&amp;L</t>
+          <t>Alpaca paper options orders in executor.py</t>
         </is>
       </c>
       <c r="F294" s="5" t="inlineStr">
         <is>
-          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
+          <t>executor.py has zero options code (equity brackets only); Alpaca SDK supports OptionLegRequest/GetOptionContractsRequest.</t>
         </is>
       </c>
       <c r="G294" s="5" t="inlineStr">
         <is>
-          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
+          <t>Construct+submit single + vertical OptionLegRequest in executor.py, PAPER only behind the config.alpaca.paper hard guard. Never live (feedback_paper_only_automation).</t>
         </is>
       </c>
       <c r="H294" s="2" t="inlineStr"/>
@@ -16907,7 +16907,7 @@
       </c>
       <c r="M294" s="3" t="inlineStr">
         <is>
-          <t>635ae960f</t>
+          <t>9c3a2a58d</t>
         </is>
       </c>
       <c r="N294" s="8" t="inlineStr"/>
@@ -16918,7 +16918,7 @@
       </c>
       <c r="B295" s="3" t="inlineStr">
         <is>
-          <t>OPT-PAPER-5</t>
+          <t>OPT-PAPER-4</t>
         </is>
       </c>
       <c r="C295" s="10" t="inlineStr">
@@ -16933,17 +16933,17 @@
       </c>
       <c r="E295" s="6" t="inlineStr">
         <is>
-          <t>Options-specific exits</t>
+          <t>Options position tracking + contract P&amp;L</t>
         </is>
       </c>
       <c r="F295" s="5" t="inlineStr">
         <is>
-          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
+          <t>Portfolio tracker is share-P&amp;L only; can't track premium/Greeks/theta/DTE.</t>
         </is>
       </c>
       <c r="G295" s="5" t="inlineStr">
         <is>
-          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
+          <t>Extend portfolio tracker for contracts: premium, Greeks, theta decay, IV, DTE, mark-to-market.</t>
         </is>
       </c>
       <c r="H295" s="2" t="inlineStr"/>
@@ -16966,13 +16966,13 @@
       </c>
       <c r="N295" s="8" t="inlineStr"/>
     </row>
-    <row r="296" ht="120" customHeight="1">
+    <row r="296" ht="45" customHeight="1">
       <c r="A296" s="2" t="n">
         <v>295</v>
       </c>
       <c r="B296" s="3" t="inlineStr">
         <is>
-          <t>UI-STRAT-1</t>
+          <t>OPT-PAPER-5</t>
         </is>
       </c>
       <c r="C296" s="10" t="inlineStr">
@@ -16982,22 +16982,22 @@
       </c>
       <c r="D296" s="5" t="inlineStr">
         <is>
-          <t>Strategy Lab</t>
+          <t>Strategy / Options Paper</t>
         </is>
       </c>
       <c r="E296" s="6" t="inlineStr">
         <is>
-          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
+          <t>Options-specific exits</t>
         </is>
       </c>
       <c r="F296" s="5" t="inlineStr">
         <is>
-          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
+          <t>Equity exits are price-stop only; options need IV/theta/expiry-aware exits.</t>
         </is>
       </c>
       <c r="G296" s="5" t="inlineStr">
         <is>
-          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
+          <t>IV-crush-around-earnings rule, time-stop before expiry, profit-take on the CONTRACT not the underlying, assignment handling.</t>
         </is>
       </c>
       <c r="H296" s="2" t="inlineStr"/>
@@ -17010,23 +17010,23 @@
       </c>
       <c r="L296" s="2" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="M296" s="3" t="inlineStr">
         <is>
-          <t>93ec11842</t>
+          <t>635ae960f</t>
         </is>
       </c>
       <c r="N296" s="8" t="inlineStr"/>
     </row>
-    <row r="297" ht="60" customHeight="1">
+    <row r="297" ht="120" customHeight="1">
       <c r="A297" s="2" t="n">
         <v>296</v>
       </c>
       <c r="B297" s="3" t="inlineStr">
         <is>
-          <t>TE-SESSION-CACHE</t>
+          <t>UI-STRAT-1</t>
         </is>
       </c>
       <c r="C297" s="10" t="inlineStr">
@@ -17036,22 +17036,22 @@
       </c>
       <c r="D297" s="5" t="inlineStr">
         <is>
-          <t>Structural Targets</t>
+          <t>Strategy Lab</t>
         </is>
       </c>
       <c r="E297" s="6" t="inlineStr">
         <is>
-          <t>Session-date cache invalidation</t>
+          <t>13-section HF cockpit rebuild + live setup_stats wiring</t>
         </is>
       </c>
       <c r="F297" s="5" t="inlineStr">
         <is>
-          <t>target_engine cache used 12h wall-clock TTL → expired mid-session (15:00-19:30 PT dead-zone) causing on-demand recomputes on tab open</t>
+          <t>Old Strategy Lab was 4-section table with fake numbers and 3x3 correlation. Didn't match 20yr HF analyst standard (no capital allocation cascade, no Wilson CI on PF, no edge-erosion radar, no BT vs Live divergence, no auto-quarantine surface).</t>
         </is>
       </c>
       <c r="G297" s="5" t="inlineStr">
         <is>
-          <t>Switched _cache_is_fresh to session-date keying (_latest_completed_session) + 36h backstop + legacy grandfather; _cache_write stamps session_date. 0 added EODHD, recompute only on new daily bar.</t>
+          <t>Rebuilt renderStrategies in kairos.html with 13 sections: portfolio cockpit, setup-family perf (LIVE from setup_stats.json with Wilson bars + PF haircut), edge erosion radar, BT vs Live divergence (surfaces PEAD canary BT 2.04 vs live 0.88), phase promotion ledger, regime×sleeve grid 8x4, correlation 8x8 + eigenvalue λ₁, sleeve interaction overlap, recent picks roster, auto-quarantine surface, mechanism+falsifier, playbook, pre-mortem. async _stratLabPatch() fetches live data.</t>
         </is>
       </c>
       <c r="H297" s="2" t="inlineStr"/>
@@ -17064,12 +17064,12 @@
       </c>
       <c r="L297" s="2" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="M297" s="3" t="inlineStr">
         <is>
-          <t>33146be5e</t>
+          <t>93ec11842</t>
         </is>
       </c>
       <c r="N297" s="8" t="inlineStr"/>
@@ -17080,7 +17080,7 @@
       </c>
       <c r="B298" s="3" t="inlineStr">
         <is>
-          <t>TE-STRATEGY-MODE</t>
+          <t>TE-SESSION-CACHE</t>
         </is>
       </c>
       <c r="C298" s="10" t="inlineStr">
@@ -17090,22 +17090,22 @@
       </c>
       <c r="D298" s="5" t="inlineStr">
         <is>
-          <t>Target Engine</t>
+          <t>Structural Targets</t>
         </is>
       </c>
       <c r="E298" s="6" t="inlineStr">
         <is>
-          <t>_strategy_mode read but never written</t>
+          <t>Session-date cache invalidation</t>
         </is>
       </c>
       <c r="F298" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
+          <t>target_engine cache used 12h wall-clock TTL → expired mid-session (15:00-19:30 PT dead-zone) causing on-demand recomputes on tab open</t>
         </is>
       </c>
       <c r="G298" s="5" t="inlineStr">
         <is>
-          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
+          <t>Switched _cache_is_fresh to session-date keying (_latest_completed_session) + 36h backstop + legacy grandfather; _cache_write stamps session_date. 0 added EODHD, recompute only on new daily bar.</t>
         </is>
       </c>
       <c r="H298" s="2" t="inlineStr"/>
@@ -17118,23 +17118,23 @@
       </c>
       <c r="L298" s="2" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="M298" s="3" t="inlineStr">
         <is>
-          <t>15f8f9600</t>
+          <t>33146be5e</t>
         </is>
       </c>
       <c r="N298" s="8" t="inlineStr"/>
     </row>
-    <row r="299" ht="105" customHeight="1">
+    <row r="299" ht="60" customHeight="1">
       <c r="A299" s="2" t="n">
         <v>298</v>
       </c>
       <c r="B299" s="3" t="inlineStr">
         <is>
-          <t>TRACKER-BUY-FILTER</t>
+          <t>TE-STRATEGY-MODE</t>
         </is>
       </c>
       <c r="C299" s="10" t="inlineStr">
@@ -17144,31 +17144,27 @@
       </c>
       <c r="D299" s="5" t="inlineStr">
         <is>
-          <t>Tracker/Feedback Loop</t>
+          <t>Target Engine</t>
         </is>
       </c>
       <c r="E299" s="6" t="inlineStr">
         <is>
-          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
+          <t>_strategy_mode read but never written</t>
         </is>
       </c>
       <c r="F299" s="5" t="inlineStr">
         <is>
-          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
+          <t>compute_trade_plan structural override read config['_strategy_mode'] which is set nowhere → override always ran mode=swing, silently mis-targeting any position/invest plan routed through it</t>
         </is>
       </c>
       <c r="G299" s="5" t="inlineStr">
         <is>
-          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+          <t>promoted to discoverable strategy_mode='swing' kwarg on compute_trade_plan; config injection still wins (mirrors _regime_name convention); behavior-neutral today</t>
         </is>
       </c>
       <c r="H299" s="2" t="inlineStr"/>
       <c r="I299" s="5" t="inlineStr"/>
-      <c r="J299" s="5" t="inlineStr">
-        <is>
-          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
-        </is>
-      </c>
+      <c r="J299" s="5" t="inlineStr"/>
       <c r="K299" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17176,27 +17172,23 @@
       </c>
       <c r="L299" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="M299" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N299" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
-        </is>
-      </c>
-    </row>
-    <row r="300" ht="135" customHeight="1">
+          <t>15f8f9600</t>
+        </is>
+      </c>
+      <c r="N299" s="8" t="inlineStr"/>
+    </row>
+    <row r="300" ht="105" customHeight="1">
       <c r="A300" s="2" t="n">
         <v>299</v>
       </c>
       <c r="B300" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
+          <t>TRACKER-BUY-FILTER</t>
         </is>
       </c>
       <c r="C300" s="10" t="inlineStr">
@@ -17206,37 +17198,29 @@
       </c>
       <c r="D300" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Tracker/Feedback Loop</t>
         </is>
       </c>
       <c r="E300" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>tracker.compute_stats_by_setup should filter to verdict='BUY' only</t>
         </is>
       </c>
       <c r="F300" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>Currently reads all closed trades from picks_history.json (627: 304 BUY + 315 WATCH + 5 None + 3 SHORT, total WR 61.2%). The tracker drives apply_setup_wr_multiplier which scales future BUY scores. Learning from WATCH/SHORT outcomes (signals the system never took) biases multipliers in non-actionable directions.</t>
         </is>
       </c>
       <c r="G300" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
-        </is>
-      </c>
-      <c r="H300" s="2" t="inlineStr">
-        <is>
-          <t>1-2 hrs</t>
-        </is>
-      </c>
-      <c r="I300" s="5" t="inlineStr">
-        <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
-        </is>
-      </c>
+          <t>Add _accepted_verdicts={'BUY'} filter at tracker.py:765 area. CAVEAT: cuts available sample sizes drastically (most setup x regime cells drop to n&lt;5 → mult=1.0). Could remove existing boosts. Verify with backtest before shipping.</t>
+        </is>
+      </c>
+      <c r="H300" s="2" t="inlineStr"/>
+      <c r="I300" s="5" t="inlineStr"/>
       <c r="J300" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+          <t>tracker.compute_stats_by_setup now filters trades to verdict in {BUY, SHORT}, excluding WATCH-stage outcomes. 689 total → 344 BUY-only. IMPORTANT downstream finding: BUY-only data shows Variant F+ may be redundant — Near-VCP/Squeeze/Pocket setups have only n=1-2 actual BUY trades in bull regime (live picks_history), vs the n=8-13 from F1+F2 backtest simulation. Variant F+ does not hurt but may not be needed; revisit after fresh data.</t>
         </is>
       </c>
       <c r="K300" s="12" t="inlineStr">
@@ -17246,27 +17230,27 @@
       </c>
       <c r="L300" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M300" s="3" t="inlineStr">
         <is>
-          <t>42c36ef91</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N300" s="8" t="inlineStr">
         <is>
-          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="301" ht="45" customHeight="1">
+          <t>python3 -c 'import tracker; s = tracker.compute_stats_by_setup(); print(s["total_trades"])' returns BUY-only count (filters WATCH).</t>
+        </is>
+      </c>
+    </row>
+    <row r="301" ht="135" customHeight="1">
       <c r="A301" s="2" t="n">
         <v>300</v>
       </c>
       <c r="B301" s="3" t="inlineStr">
         <is>
-          <t>STOCKSMITH-BOOK-RISK</t>
+          <t>MOD-1</t>
         </is>
       </c>
       <c r="C301" s="10" t="inlineStr">
@@ -17276,27 +17260,39 @@
       </c>
       <c r="D301" s="5" t="inlineStr">
         <is>
-          <t>V2 Dashboard / Risk</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E301" s="6" t="inlineStr">
         <is>
-          <t>Book Risk surface + per-lens analytics (§6)</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F301" s="5" t="inlineStr">
         <is>
-          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G301" s="5" t="inlineStr">
         <is>
-          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
-        </is>
-      </c>
-      <c r="H301" s="2" t="inlineStr"/>
-      <c r="I301" s="5" t="inlineStr"/>
-      <c r="J301" s="5" t="inlineStr"/>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+        </is>
+      </c>
+      <c r="H301" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I301" s="5" t="inlineStr">
+        <is>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
+        </is>
+      </c>
+      <c r="J301" s="5" t="inlineStr">
+        <is>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+        </is>
+      </c>
       <c r="K301" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17304,23 +17300,27 @@
       </c>
       <c r="L301" s="2" t="inlineStr">
         <is>
-          <t>2026-05-30</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M301" s="3" t="inlineStr">
         <is>
-          <t>50cace567</t>
-        </is>
-      </c>
-      <c r="N301" s="8" t="inlineStr"/>
-    </row>
-    <row r="302" ht="120" customHeight="1">
+          <t>42c36ef91</t>
+        </is>
+      </c>
+      <c r="N301" s="8" t="inlineStr">
+        <is>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="302" ht="45" customHeight="1">
       <c r="A302" s="2" t="n">
         <v>301</v>
       </c>
       <c r="B302" s="3" t="inlineStr">
         <is>
-          <t>RECENCY-FLOOR</t>
+          <t>STOCKSMITH-BOOK-RISK</t>
         </is>
       </c>
       <c r="C302" s="10" t="inlineStr">
@@ -17330,31 +17330,27 @@
       </c>
       <c r="D302" s="5" t="inlineStr">
         <is>
-          <t>Validation Hygiene</t>
+          <t>V2 Dashboard / Risk</t>
         </is>
       </c>
       <c r="E302" s="6" t="inlineStr">
         <is>
-          <t>_validations needs recency floor — auto-revert stale boosts</t>
+          <t>Book Risk surface + per-lens analytics (§6)</t>
         </is>
       </c>
       <c r="F302" s="5" t="inlineStr">
         <is>
-          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
+          <t>Book Risk (exposure/Greeks/optimizer/attribution/crowding/hedge) + VaR mode-aware + DCF grid + Earnings whisper; honest dashes</t>
         </is>
       </c>
       <c r="G302" s="5" t="inlineStr">
         <is>
-          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
+          <t>Stocksmith.html BookRiskPanel + InvDcfSensitivity + EoWhisperRevisions</t>
         </is>
       </c>
       <c r="H302" s="2" t="inlineStr"/>
       <c r="I302" s="5" t="inlineStr"/>
-      <c r="J302" s="5" t="inlineStr">
-        <is>
-          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
-        </is>
-      </c>
+      <c r="J302" s="5" t="inlineStr"/>
       <c r="K302" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17362,27 +17358,23 @@
       </c>
       <c r="L302" s="2" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-30</t>
         </is>
       </c>
       <c r="M302" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
-        </is>
-      </c>
-      <c r="N302" s="8" t="inlineStr">
-        <is>
-          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
-        </is>
-      </c>
-    </row>
-    <row r="303" ht="60" customHeight="1">
+          <t>50cace567</t>
+        </is>
+      </c>
+      <c r="N302" s="8" t="inlineStr"/>
+    </row>
+    <row r="303" ht="120" customHeight="1">
       <c r="A303" s="2" t="n">
         <v>302</v>
       </c>
       <c r="B303" s="3" t="inlineStr">
         <is>
-          <t>MOMENTUM-TAB</t>
+          <t>RECENCY-FLOOR</t>
         </is>
       </c>
       <c r="C303" s="10" t="inlineStr">
@@ -17392,27 +17384,31 @@
       </c>
       <c r="D303" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Momentum</t>
+          <t>Validation Hygiene</t>
         </is>
       </c>
       <c r="E303" s="6" t="inlineStr">
         <is>
-          <t>New 🚀 Momentum workspace tab</t>
+          <t>_validations needs recency floor — auto-revert stale boosts</t>
         </is>
       </c>
       <c r="F303" s="5" t="inlineStr">
         <is>
-          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
+          <t>Current setup_score_multiplier._validations gates on lifetime n&gt;=30 + wr_lb&lt;0.30 for demotions but NO gate for boosts. Stale boost evidence (e.g., 10W Pullback 1.5x backed by n=87 / WR 73.6% historical) can amplify a strategy that has been losing recently (last 11 BUYs: 9.1% WR, -5.31% avg). Bug class only surfaced because of the CAR target1 catastrophe.</t>
         </is>
       </c>
       <c r="G303" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
+          <t>Add recency check: when a boost (mult &gt; 1.0) is configured, require the LAST N=20 closed signals for (setup x regime) to clear wr_lb &gt;= 0.40. If not, silently revert to 1.0 (no boost). Same pattern as existing demotion gate at analysis.py:8846. Defer until BUY-only filter discussion is resolved (TRACKER-BUY-FILTER).</t>
         </is>
       </c>
       <c r="H303" s="2" t="inlineStr"/>
       <c r="I303" s="5" t="inlineStr"/>
-      <c r="J303" s="5" t="inlineStr"/>
+      <c r="J303" s="5" t="inlineStr">
+        <is>
+          <t>Implemented at analysis.py:9342 area. New _recent_setup_wr_lb() reads signal_log, takes last 20 closed signals per setup, computes Wilson 95% LB on WR. When mult &gt; 1.0 (boost) AND recent n&gt;=10 AND wr_lb&lt;0.40, silently revert to 1.0. Sparse recent (n&lt;10) preserves historical boost. Process-cached. VERIFIED: catches 10-Week Pullback (1.5x → 1.0x, recent wr_lb 5.2%) and VCP Breakout (1.3x → 1.0x, recent wr_lb 11.2%) — both had stale historical boosts that recency-gate correctly neutralizes until performance recovers.</t>
+        </is>
+      </c>
       <c r="K303" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17420,15 +17416,19 @@
       </c>
       <c r="L303" s="2" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="M303" s="3" t="inlineStr">
         <is>
-          <t>27fd646b1</t>
-        </is>
-      </c>
-      <c r="N303" s="8" t="inlineStr"/>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N303" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'from analysis import _recent_setup_wr_lb; print(_recent_setup_wr_lb("10-Week Pullback", 20))' → returns (n, wr_lb). If n&gt;=10 and wr_lb&lt;0.40, boost gets reverted.</t>
+        </is>
+      </c>
     </row>
     <row r="304" ht="60" customHeight="1">
       <c r="A304" s="2" t="n">
@@ -17436,7 +17436,7 @@
       </c>
       <c r="B304" s="3" t="inlineStr">
         <is>
-          <t>SCANNER-QUICK-PANELS</t>
+          <t>MOMENTUM-TAB</t>
         </is>
       </c>
       <c r="C304" s="10" t="inlineStr">
@@ -17446,22 +17446,22 @@
       </c>
       <c r="D304" s="5" t="inlineStr">
         <is>
-          <t>Workspaces / Signal Scanner</t>
+          <t>Workspaces / Momentum</t>
         </is>
       </c>
       <c r="E304" s="6" t="inlineStr">
         <is>
-          <t>5 quick-glance panels above watchlist table</t>
+          <t>New 🚀 Momentum workspace tab</t>
         </is>
       </c>
       <c r="F304" s="5" t="inlineStr">
         <is>
-          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
+          <t>Ranks scan universe by composite (raw_momentum_score×0.5 + sharpe_norm×0.25 + rs_rank×0.25). Filterable by setup family + grade A/B/C. Click row → detail. Sidebar count = Grade-A + composite≥80 tickers</t>
         </is>
       </c>
       <c r="G304" s="5" t="inlineStr">
         <is>
-          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+          <t>kairos.html QuantMomentum IIFE + V3_WORKSPACES.momentum + dispatcher branch</t>
         </is>
       </c>
       <c r="H304" s="2" t="inlineStr"/>
@@ -17479,60 +17479,48 @@
       </c>
       <c r="M304" s="3" t="inlineStr">
         <is>
-          <t>dfbe955fe</t>
+          <t>27fd646b1</t>
         </is>
       </c>
       <c r="N304" s="8" t="inlineStr"/>
     </row>
-    <row r="305" ht="45" customHeight="1">
+    <row r="305" ht="60" customHeight="1">
       <c r="A305" s="2" t="n">
         <v>304</v>
       </c>
       <c r="B305" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C305" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>SCANNER-QUICK-PANELS</t>
+        </is>
+      </c>
+      <c r="C305" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D305" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Workspaces / Signal Scanner</t>
         </is>
       </c>
       <c r="E305" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>5 quick-glance panels above watchlist table</t>
         </is>
       </c>
       <c r="F305" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>Top 5 AI Predictions · Fresh Entries · Top Momentum · Earnings This Week · Volume Surges. Each panel uses shared _qpCard + _qpFrame helpers. Click row → setDetailTicker (with ML cache fallback for R2000)</t>
         </is>
       </c>
       <c r="G305" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
-        </is>
-      </c>
-      <c r="H305" s="2" t="inlineStr">
-        <is>
-          <t>verified</t>
-        </is>
-      </c>
-      <c r="I305" s="5" t="inlineStr">
-        <is>
-          <t>Win: persistence works; no silent overwrites.</t>
-        </is>
-      </c>
-      <c r="J305" s="5" t="inlineStr">
-        <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
-        </is>
-      </c>
+          <t>kairos.html QuantScanner.renderQuickPanels + panelXxx helpers + .qs-quick-* CSS</t>
+        </is>
+      </c>
+      <c r="H305" s="2" t="inlineStr"/>
+      <c r="I305" s="5" t="inlineStr"/>
+      <c r="J305" s="5" t="inlineStr"/>
       <c r="K305" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17540,15 +17528,15 @@
       </c>
       <c r="L305" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M305" s="3" t="inlineStr"/>
-      <c r="N305" s="8" t="inlineStr">
-        <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="M305" s="3" t="inlineStr">
+        <is>
+          <t>dfbe955fe</t>
+        </is>
+      </c>
+      <c r="N305" s="8" t="inlineStr"/>
     </row>
     <row r="306" ht="45" customHeight="1">
       <c r="A306" s="2" t="n">
@@ -17556,7 +17544,7 @@
       </c>
       <c r="B306" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
+          <t>B4</t>
         </is>
       </c>
       <c r="C306" s="13" t="inlineStr">
@@ -17571,32 +17559,32 @@
       </c>
       <c r="E306" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F306" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G306" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H306" s="2" t="inlineStr">
         <is>
-          <t>verified (no change needed)</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I306" s="5" t="inlineStr">
         <is>
-          <t>Win: confirms infrastructure still healthy.</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J306" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
         </is>
       </c>
       <c r="K306" s="12" t="inlineStr">
@@ -17612,7 +17600,7 @@
       <c r="M306" s="3" t="inlineStr"/>
       <c r="N306" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
         </is>
       </c>
     </row>
@@ -17622,7 +17610,7 @@
       </c>
       <c r="B307" s="3" t="inlineStr">
         <is>
-          <t>UI-3</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C307" s="13" t="inlineStr">
@@ -17632,35 +17620,39 @@
       </c>
       <c r="D307" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E307" s="6" t="inlineStr">
         <is>
-          <t>Remove emoji icons from Thesis + Research labels</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F307" s="5" t="inlineStr">
         <is>
-          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G307" s="5" t="inlineStr">
         <is>
-          <t>Removed emojis from FD sub-tab nav + section headers.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H307" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I307" s="5" t="inlineStr">
         <is>
-          <t>Low / cosmetic</t>
-        </is>
-      </c>
-      <c r="J307" s="5" t="inlineStr"/>
+          <t>Win: confirms infrastructure still healthy.</t>
+        </is>
+      </c>
+      <c r="J307" s="5" t="inlineStr">
+        <is>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
       <c r="K307" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -17668,17 +17660,13 @@
       </c>
       <c r="L307" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
-      <c r="M307" s="3" t="inlineStr">
-        <is>
-          <t>24fd7c273</t>
-        </is>
-      </c>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M307" s="3" t="inlineStr"/>
       <c r="N307" s="8" t="inlineStr">
         <is>
-          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
         </is>
       </c>
     </row>
@@ -17688,59 +17676,63 @@
       </c>
       <c r="B308" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
-        </is>
-      </c>
-      <c r="C308" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>UI-3</t>
+        </is>
+      </c>
+      <c r="C308" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D308" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>UI</t>
         </is>
       </c>
       <c r="E308" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Remove emoji icons from Thesis + Research labels</t>
         </is>
       </c>
       <c r="F308" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Thesis and Research labels had emoji icons; user wanted plain.</t>
         </is>
       </c>
       <c r="G308" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+          <t>Removed emojis from FD sub-tab nav + section headers.</t>
         </is>
       </c>
       <c r="H308" s="2" t="inlineStr">
         <is>
-          <t>5 min after answer</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I308" s="5" t="inlineStr">
         <is>
-          <t>Win: -671 lines.</t>
-        </is>
-      </c>
-      <c r="J308" s="5" t="inlineStr">
-        <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K308" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L308" s="2" t="inlineStr"/>
-      <c r="M308" s="3" t="inlineStr"/>
+          <t>Low / cosmetic</t>
+        </is>
+      </c>
+      <c r="J308" s="5" t="inlineStr"/>
+      <c r="K308" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L308" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M308" s="3" t="inlineStr">
+        <is>
+          <t>24fd7c273</t>
+        </is>
+      </c>
       <c r="N308" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>Open elite-detail - tabs show "Thesis" and "Research" without emojis.</t>
         </is>
       </c>
     </row>
@@ -17750,7 +17742,7 @@
       </c>
       <c r="B309" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
+          <t>CLEAN-2</t>
         </is>
       </c>
       <c r="C309" s="10" t="inlineStr">
@@ -17760,37 +17752,37 @@
       </c>
       <c r="D309" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E309" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
         </is>
       </c>
       <c r="F309" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
         </is>
       </c>
       <c r="G309" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
         </is>
       </c>
       <c r="H309" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>5 min after answer</t>
         </is>
       </c>
       <c r="I309" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Win: -671 lines.</t>
         </is>
       </c>
       <c r="J309" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
+          <t>Standard data-migration retention practice.</t>
         </is>
       </c>
       <c r="K309" s="14" t="inlineStr">
@@ -17812,109 +17804,109 @@
       </c>
       <c r="B310" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C310" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C310" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D310" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E310" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
         </is>
       </c>
       <c r="F310" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
         </is>
       </c>
       <c r="G310" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
         </is>
       </c>
       <c r="H310" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>hours-days each</t>
         </is>
       </c>
       <c r="I310" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win varies; defer until PERF-7 measured.</t>
         </is>
       </c>
       <c r="J310" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K310" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K310" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="L310" s="2" t="inlineStr"/>
       <c r="M310" s="3" t="inlineStr"/>
       <c r="N310" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="311" ht="75" customHeight="1">
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="311" ht="45" customHeight="1">
       <c r="A311" s="2" t="n">
         <v>310</v>
       </c>
       <c r="B311" s="3" t="inlineStr">
         <is>
-          <t>MOD-2</t>
-        </is>
-      </c>
-      <c r="C311" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C311" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D311" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E311" s="6" t="inlineStr">
         <is>
-          <t>Pixel-diff regression baseline</t>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
         </is>
       </c>
       <c r="F311" s="5" t="inlineStr">
         <is>
-          <t>After modularization, no automated visual-regression catch.</t>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
         </is>
       </c>
       <c r="G311" s="5" t="inlineStr">
         <is>
-          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
         </is>
       </c>
       <c r="H311" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I311" s="5" t="inlineStr">
         <is>
-          <t>Win: catches accidental layout regressions.</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J311" s="5" t="inlineStr">
         <is>
-          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+          <t>Agents skim and miss post-filter subset analysis.</t>
         </is>
       </c>
       <c r="K311" s="15" t="inlineStr">
@@ -17922,147 +17914,209 @@
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L311" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-11</t>
-        </is>
-      </c>
+      <c r="L311" s="2" t="inlineStr"/>
       <c r="M311" s="3" t="inlineStr"/>
       <c r="N311" s="8" t="inlineStr">
         <is>
-          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="312" ht="195" customHeight="1">
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="312" ht="75" customHeight="1">
       <c r="A312" s="2" t="n">
         <v>311</v>
       </c>
       <c r="B312" s="3" t="inlineStr">
         <is>
+          <t>MOD-2</t>
+        </is>
+      </c>
+      <c r="C312" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="D312" s="5" t="inlineStr">
+        <is>
+          <t>UI / Modularization</t>
+        </is>
+      </c>
+      <c r="E312" s="6" t="inlineStr">
+        <is>
+          <t>Pixel-diff regression baseline</t>
+        </is>
+      </c>
+      <c r="F312" s="5" t="inlineStr">
+        <is>
+          <t>After modularization, no automated visual-regression catch.</t>
+        </is>
+      </c>
+      <c r="G312" s="5" t="inlineStr">
+        <is>
+          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+        </is>
+      </c>
+      <c r="H312" s="2" t="inlineStr">
+        <is>
+          <t>2-3 hrs</t>
+        </is>
+      </c>
+      <c r="I312" s="5" t="inlineStr">
+        <is>
+          <t>Win: catches accidental layout regressions.</t>
+        </is>
+      </c>
+      <c r="J312" s="5" t="inlineStr">
+        <is>
+          <t>User declared out of scope 2026-05-11. Pixel-diff regression testing not needed; visual regressions can be caught by manual review when CSS/markup changes ship. Test scaffold remains in tests/04-pixel-diff.spec.js for future opt-in but no baseline PNGs will be generated.</t>
+        </is>
+      </c>
+      <c r="K312" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L312" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="M312" s="3" t="inlineStr"/>
+      <c r="N312" s="8" t="inlineStr">
+        <is>
+          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313" ht="195" customHeight="1">
+      <c r="A313" s="2" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
           <t>OB-CONFLUENCE-PROPOSAL-REJECTED</t>
         </is>
       </c>
-      <c r="C312" s="10" t="inlineStr">
+      <c r="C313" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="D312" s="5" t="inlineStr">
+      <c r="D313" s="5" t="inlineStr">
         <is>
           <t>Signals / Cross-Check</t>
         </is>
       </c>
-      <c r="E312" s="6" t="inlineStr">
+      <c r="E313" s="6" t="inlineStr">
         <is>
           <t>OB-confluence Wilson bump + OB-aware stop — proposals KILLED by backtest evidence</t>
         </is>
       </c>
-      <c r="F312" s="5" t="inlineStr">
+      <c r="F313" s="5" t="inlineStr">
         <is>
           <t>User asked 2026-05-12 to ship #2 (Wilson-bump score factor for bullish OB confluence within 5% of entry) and #5 (OB-low as stop instead of 1.25xATR). Per Principle 1 / Principle 7, ran post-hoc validation: scripts/validate_ob_confluence.py retroactively tags every closed trade from existing portfolio_backtest outputs with SMC state at entry date, computes Wilson 95% LB per subset.
 RESULT (750-day backtest · n=384): Bull OB confluence within 5% of entry DECREASES Wilson LB by -8.6pp (14.6% vs baseline 23.1%). BOS-bullish boost: -3.4pp. SMC-bullish direction boost: -3.6pp. Per #5 simulation, 35 of 39 (90%) OB-low-as-stop would have loosened the stop; 25 of those still ended in losses (looser stops do not rescue broken setups, they extend exposure).
 Principle 4 fires: proposals FALSIFIED, killed permanently (not retuned). Doing the change without this validation would have introduced a 6-9pp Wilson-LB drag on every BUY signal.</t>
         </is>
       </c>
-      <c r="G312" s="5" t="inlineStr">
+      <c r="G313" s="5" t="inlineStr">
         <is>
           <t>Built scripts/validate_ob_confluence.py to retroactively run smart_money.score_smc() on the historical OHLCV at each trade's entry date, tag with OB-confluence + BOS + CHoCH flags, compute Wilson 95% LB per subset, and apply Principle 1 gates (n&gt;=30, lift&gt;=5pp). Cross-validated on 250d (n=142) and 750d (n=384) backtest outputs. Both agree: NO EDGE.</t>
         </is>
       </c>
-      <c r="H312" s="2" t="inlineStr">
+      <c r="H313" s="2" t="inlineStr">
         <is>
           <t>Days of work avoided (would have shipped a degrading change).</t>
         </is>
       </c>
-      <c r="I312" s="5" t="inlineStr">
+      <c r="I313" s="5" t="inlineStr">
         <is>
           <t>Mechanism (Principle 2): institutional OBs are supposed to mark re-add zones for smart money. Falsification (Principle 4): if the data doesn't show OB-confluent trades winning more, the mechanism either doesn't exist for retail-accessible OB detection at daily resolution OR is already priced into our 5-pillar score. Either way: ship nothing. The proposals are dead. Win: prevented a 6-9pp Wilson-LB drag from being added to live scoring. Lost: nothing — we didn't change live scoring, no opportunity cost.</t>
         </is>
       </c>
-      <c r="J312" s="5" t="inlineStr">
+      <c r="J313" s="5" t="inlineStr">
         <is>
           <t>Validator script is reusable infrastructure. Re-run any time the SMC detection logic or score thresholds change. NOTE: baseline WR in 750d backtest is 27.3% (low) — the absolute level reflects backtest-window-specific market conditions; the SUBSET comparisons are valid regardless because they share the same baseline. Do not interpret 23.1% Wilson LB as a system-level edge — that's a separate question. This validation answers ONLY: does OB-confluence improve selection within whatever the system already does.</t>
         </is>
       </c>
-      <c r="K312" s="15" t="inlineStr">
+      <c r="K313" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="L312" s="2" t="inlineStr">
+      <c r="L313" s="2" t="inlineStr">
         <is>
           <t>2026-05-12</t>
-        </is>
-      </c>
-      <c r="M312" s="3" t="inlineStr"/>
-      <c r="N312" s="8" t="inlineStr">
-        <is>
-          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="313" ht="90" customHeight="1">
-      <c r="A313" s="2" t="n">
-        <v>312</v>
-      </c>
-      <c r="B313" s="3" t="inlineStr">
-        <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C313" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
-        </is>
-      </c>
-      <c r="D313" s="5" t="inlineStr">
-        <is>
-          <t>Data / Universe</t>
-        </is>
-      </c>
-      <c r="E313" s="6" t="inlineStr">
-        <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
-        </is>
-      </c>
-      <c r="F313" s="5" t="inlineStr">
-        <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
-        </is>
-      </c>
-      <c r="G313" s="5" t="inlineStr">
-        <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
-        </is>
-      </c>
-      <c r="H313" s="2" t="inlineStr">
-        <is>
-          <t>$$ + 1 day</t>
-        </is>
-      </c>
-      <c r="I313" s="5" t="inlineStr">
-        <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
-        </is>
-      </c>
-      <c r="J313" s="5" t="inlineStr">
-        <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K313" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L313" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M313" s="3" t="inlineStr"/>
       <c r="N313" s="8" t="inlineStr">
+        <is>
+          <t>python3 scripts/validate_ob_confluence.py --backtest cache/portfolio_backtest_750d_20260509_100501.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="314" ht="90" customHeight="1">
+      <c r="A314" s="2" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C314" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D314" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E314" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F314" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G314" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H314" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I314" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J314" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K314" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L314" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M314" s="3" t="inlineStr"/>
+      <c r="N314" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -18167,10 +18221,10 @@
         <v>90</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5">
@@ -18224,10 +18278,10 @@
         <v>115</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
   </sheetData>

</xml_diff>